<commit_message>
hardware(bom): refresh controlled workbook
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdf8aa1c97d914cda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R7fbafd8b97484465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R09e9eb8e4ee0464d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R64fda1d17d7d4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R755664bb53cf48f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R8096d1c63b444833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rbeb8778db6b14863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R1363689b07f944eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -487,7 +487,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -497,7 +497,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -508,7 +508,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -519,7 +519,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -529,7 +529,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -540,7 +540,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -551,7 +551,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -985,7 +985,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>d8f938fa8397</x:v>
+        <x:v>9ac919161d2f</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1063,10 +1063,10 @@
         <x:v>Engineering and supplier selections</x:v>
       </x:c>
       <x:c r="B23" s="72" t="str">
-        <x:v>U8, PWR-TVS-01, PWR-FUSE-01, HSG-VC</x:v>
+        <x:v>PWR-TVS-01, PWR-FUSE-01, HSG-VC</x:v>
       </x:c>
       <x:c r="C23" s="73" t="str">
-        <x:v>Close regional modem identity, surge/fuse coordination and housing FAI supplier</x:v>
+        <x:v>Close surge/fuse coordination and housing FAI supplier release</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3355,10 +3355,10 @@
         <x:v>SCALE_CEIL_FROM_20_BASELINE</x:v>
       </x:c>
       <x:c r="V30" s="14" t="str">
-        <x:v>BLOCKED_ENGINEERING_SELECTION</x:v>
+        <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W30" s="14" t="str">
-        <x:v>SELECTED_PENDING_REGION_OPERATOR_BURST_SAMPLE</x:v>
+        <x:v>SELECTED_PENDING_INCOMING_ID_AND_POST_ASSEMBLY_EVT</x:v>
       </x:c>
       <x:c r="X30" s="17" t="str">
         <x:v>Quectel authorized channel or CM with traceability</x:v>
@@ -10488,7 +10488,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89ff2e9d8bbc4633"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583d278219624076"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11288,7 +11288,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U9" s="14" t="str">
-        <x:v>SELECTED_PENDING_REGION_OPERATOR_BURST_SAMPLE</x:v>
+        <x:v>SELECTED_PENDING_INCOMING_ID_AND_POST_ASSEMBLY_EVT</x:v>
       </x:c>
       <x:c r="V9" s="17" t="str">
         <x:v>Quectel authorized channel or CM with traceability</x:v>
@@ -11297,7 +11297,7 @@
         <x:v>IMEI label firmware RF conducted attach TLS</x:v>
       </x:c>
       <x:c r="X9" s="17" t="str">
-        <x:v>Rev.A freeze source MAIN_COMPONENT_FREEZE_REV_A.csv; blockers: exact ordered firmware/region identity; operator attach; LTE and EGPRS burst; certification; cold-limit qualification</x:v>
+        <x:v>Rev.A freeze source MAIN_COMPONENT_FREEZE_REV_A.csv; blockers: ordered module marking and firmware identity at incoming inspection; operator attach; LTE and EGPRS burst; certification; cold-limit qualification</x:v>
       </x:c>
       <x:c r="Y9" s="2" t="str"/>
       <x:c r="Z9" s="2" t="str">
@@ -11310,7 +11310,7 @@
         <x:v>-35..75 operating; -40..85 extended</x:v>
       </x:c>
       <x:c r="AC9" s="14" t="str">
-        <x:v>BLOCKED_ENGINEERING_SELECTION</x:v>
+        <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -36582,7 +36582,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcde0ebe534024918"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c6d4fdd3b8c4558"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37509,7 +37509,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdef3a100b53a49c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaaa898262eb48e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware(bom): refresh RFQ workbook traceability
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R755664bb53cf48f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R8096d1c63b444833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rbeb8778db6b14863"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R1363689b07f944eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R92a04400071047ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R570a8e38c19c40ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R87137cd7919b4b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R632e2102b1134eec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -76,6 +76,16 @@
       <x:i/>
       <x:sz val="10"/>
       <x:color rgb="FF4B5563"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -316,7 +326,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="77">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -476,6 +486,17 @@
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -631,26 +652,27 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RfqTable" displayName="RfqTable" ref="A1:R20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="18">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RfqTable" displayName="RfqTable" ref="A1:S20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="RFQ_ID"/>
-    <x:tableColumn id="2" name="Category"/>
-    <x:tableColumn id="3" name="Manufacturer"/>
-    <x:tableColumn id="4" name="MPN_or_spec"/>
-    <x:tableColumn id="5" name="Required_qty_4"/>
-    <x:tableColumn id="6" name="Required_qty_10"/>
-    <x:tableColumn id="7" name="Required_qty_20"/>
-    <x:tableColumn id="8" name="Preferred_channel"/>
-    <x:tableColumn id="9" name="Quote_date"/>
-    <x:tableColumn id="10" name="Supplier"/>
-    <x:tableColumn id="11" name="URL"/>
-    <x:tableColumn id="12" name="MOQ"/>
-    <x:tableColumn id="13" name="Lead_time_days"/>
-    <x:tableColumn id="14" name="Stock_claim"/>
-    <x:tableColumn id="15" name="Traceability_required"/>
-    <x:tableColumn id="16" name="Sample_required"/>
-    <x:tableColumn id="17" name="Status"/>
-    <x:tableColumn id="18" name="Blocking_check"/>
+    <x:tableColumn id="2" name="BOM_Item_IDs"/>
+    <x:tableColumn id="3" name="Category"/>
+    <x:tableColumn id="4" name="Manufacturer"/>
+    <x:tableColumn id="5" name="MPN_or_spec"/>
+    <x:tableColumn id="6" name="Required_qty_4"/>
+    <x:tableColumn id="7" name="Required_qty_10"/>
+    <x:tableColumn id="8" name="Required_qty_20"/>
+    <x:tableColumn id="9" name="Preferred_channel"/>
+    <x:tableColumn id="10" name="Quote_date"/>
+    <x:tableColumn id="11" name="Supplier"/>
+    <x:tableColumn id="12" name="URL"/>
+    <x:tableColumn id="13" name="MOQ"/>
+    <x:tableColumn id="14" name="Lead_time_days"/>
+    <x:tableColumn id="15" name="Stock_claim"/>
+    <x:tableColumn id="16" name="Traceability_required"/>
+    <x:tableColumn id="17" name="Sample_required"/>
+    <x:tableColumn id="18" name="Status"/>
+    <x:tableColumn id="19" name="Blocking_check"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -985,7 +1007,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>9ac919161d2f</x:v>
+        <x:v>ba7a886ccb56</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10488,7 +10510,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583d278219624076"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85bf73224a0e4c40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36582,7 +36604,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c6d4fdd3b8c4558"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b4af2bb92324d0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36591,915 +36613,976 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="34" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="15" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="15" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="38" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="26" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="11" t="str">
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="79" t="str">
         <x:v>RFQ_ID</x:v>
       </x:c>
-      <x:c r="B1" s="12" t="str">
+      <x:c r="B1" s="79" t="str">
+        <x:v>BOM_Item_IDs</x:v>
+      </x:c>
+      <x:c r="C1" s="79" t="str">
         <x:v>Category</x:v>
       </x:c>
-      <x:c r="C1" s="12" t="str">
+      <x:c r="D1" s="79" t="str">
         <x:v>Manufacturer</x:v>
       </x:c>
-      <x:c r="D1" s="12" t="str">
+      <x:c r="E1" s="79" t="str">
         <x:v>MPN_or_spec</x:v>
       </x:c>
-      <x:c r="E1" s="12" t="str">
+      <x:c r="F1" s="79" t="str">
         <x:v>Required_qty_4</x:v>
       </x:c>
-      <x:c r="F1" s="12" t="str">
+      <x:c r="G1" s="79" t="str">
         <x:v>Required_qty_10</x:v>
       </x:c>
-      <x:c r="G1" s="12" t="str">
+      <x:c r="H1" s="79" t="str">
         <x:v>Required_qty_20</x:v>
       </x:c>
-      <x:c r="H1" s="12" t="str">
+      <x:c r="I1" s="79" t="str">
         <x:v>Preferred_channel</x:v>
       </x:c>
-      <x:c r="I1" s="12" t="str">
+      <x:c r="J1" s="79" t="str">
         <x:v>Quote_date</x:v>
       </x:c>
-      <x:c r="J1" s="12" t="str">
+      <x:c r="K1" s="79" t="str">
         <x:v>Supplier</x:v>
       </x:c>
-      <x:c r="K1" s="12" t="str">
+      <x:c r="L1" s="79" t="str">
         <x:v>URL</x:v>
       </x:c>
-      <x:c r="L1" s="12" t="str">
+      <x:c r="M1" s="79" t="str">
         <x:v>MOQ</x:v>
       </x:c>
-      <x:c r="M1" s="12" t="str">
+      <x:c r="N1" s="79" t="str">
         <x:v>Lead_time_days</x:v>
       </x:c>
-      <x:c r="N1" s="12" t="str">
+      <x:c r="O1" s="79" t="str">
         <x:v>Stock_claim</x:v>
       </x:c>
-      <x:c r="O1" s="12" t="str">
+      <x:c r="P1" s="79" t="str">
         <x:v>Traceability_required</x:v>
       </x:c>
-      <x:c r="P1" s="12" t="str">
+      <x:c r="Q1" s="79" t="str">
         <x:v>Sample_required</x:v>
       </x:c>
-      <x:c r="Q1" s="12" t="str">
+      <x:c r="R1" s="79" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="R1" s="13" t="str">
+      <x:c r="S1" s="79" t="str">
         <x:v>Blocking_check</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="2" t="str">
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2" s="81" t="str">
         <x:v>RFQ-001</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="str">
+      <x:c r="B2" s="81" t="str">
+        <x:v>U1</x:v>
+      </x:c>
+      <x:c r="C2" s="81" t="str">
         <x:v>MCU</x:v>
       </x:c>
-      <x:c r="C2" s="2" t="str">
+      <x:c r="D2" s="81" t="str">
         <x:v>STMicroelectronics</x:v>
       </x:c>
-      <x:c r="D2" s="14" t="str">
+      <x:c r="E2" s="81" t="str">
         <x:v>STM32U585VIT6Q</x:v>
       </x:c>
-      <x:c r="E2" s="16" t="n">
+      <x:c r="F2" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F2" s="16" t="n">
+      <x:c r="G2" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G2" s="16" t="n">
+      <x:c r="H2" s="81" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H2" s="2" t="str">
+      <x:c r="I2" s="81" t="str">
         <x:v>Authorized distributor</x:v>
       </x:c>
-      <x:c r="I2" s="2" t="str"/>
-      <x:c r="J2" s="2" t="str"/>
-      <x:c r="K2" s="2" t="str"/>
-      <x:c r="L2" s="16" t="str"/>
-      <x:c r="M2" s="16" t="str"/>
-      <x:c r="N2" s="2" t="str"/>
-      <x:c r="O2" s="2" t="str">
+      <x:c r="J2" s="81"/>
+      <x:c r="K2" s="81"/>
+      <x:c r="L2" s="81"/>
+      <x:c r="M2" s="81"/>
+      <x:c r="N2" s="81"/>
+      <x:c r="O2" s="81"/>
+      <x:c r="P2" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P2" s="2" t="str">
+      <x:c r="Q2" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q2" s="14" t="str">
+      <x:c r="R2" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R2" s="17" t="str">
+      <x:c r="S2" s="81" t="str">
         <x:v>Package marking ID readout and exact LQFP100 package control</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="2" t="str">
+    <x:row r="3" ht="54" customHeight="1">
+      <x:c r="A3" s="81" t="str">
         <x:v>RFQ-002</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="str">
+      <x:c r="B3" s="81" t="str">
+        <x:v>MK1</x:v>
+      </x:c>
+      <x:c r="C3" s="81" t="str">
         <x:v>Microphone</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="str">
+      <x:c r="D3" s="81" t="str">
         <x:v>TDK InvenSense</x:v>
       </x:c>
-      <x:c r="D3" s="14" t="str">
+      <x:c r="E3" s="81" t="str">
         <x:v>MMICT5838-00-012 same lot</x:v>
       </x:c>
-      <x:c r="E3" s="16" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F3" s="16" t="n">
+      <x:c r="F3" s="81" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G3" s="81" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="G3" s="16" t="n">
+      <x:c r="H3" s="81" t="n">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="H3" s="2" t="str">
+      <x:c r="I3" s="81" t="str">
         <x:v>Authorized distributor</x:v>
       </x:c>
-      <x:c r="I3" s="2" t="str"/>
-      <x:c r="J3" s="2" t="str"/>
-      <x:c r="K3" s="2" t="str"/>
-      <x:c r="L3" s="16" t="str"/>
-      <x:c r="M3" s="16" t="str"/>
-      <x:c r="N3" s="2" t="str"/>
-      <x:c r="O3" s="2" t="str">
+      <x:c r="J3" s="81"/>
+      <x:c r="K3" s="81"/>
+      <x:c r="L3" s="81"/>
+      <x:c r="M3" s="81"/>
+      <x:c r="N3" s="81"/>
+      <x:c r="O3" s="81"/>
+      <x:c r="P3" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P3" s="2" t="str">
+      <x:c r="Q3" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q3" s="14" t="str">
+      <x:c r="R3" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R3" s="17" t="str">
+      <x:c r="S3" s="81" t="str">
         <x:v>Acoustic sensitivity noise phase matching and bottom-port assembly control</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="2" t="str">
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" s="81" t="str">
         <x:v>RFQ-003</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="str">
+      <x:c r="B4" s="81" t="str">
+        <x:v>U8</x:v>
+      </x:c>
+      <x:c r="C4" s="81" t="str">
         <x:v>Cellular</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="str">
+      <x:c r="D4" s="81" t="str">
         <x:v>Quectel</x:v>
       </x:c>
-      <x:c r="D4" s="14" t="str">
-        <x:v>BG95-M3 regional firmware identity</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="n">
+      <x:c r="E4" s="81" t="str">
+        <x:v>BG95-M3 marking and firmware identity</x:v>
+      </x:c>
+      <x:c r="F4" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="n">
+      <x:c r="G4" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G4" s="16" t="n">
+      <x:c r="H4" s="81" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H4" s="2" t="str">
+      <x:c r="I4" s="81" t="str">
         <x:v>Quectel authorized channel</x:v>
       </x:c>
-      <x:c r="I4" s="2" t="str"/>
-      <x:c r="J4" s="2" t="str"/>
-      <x:c r="K4" s="2" t="str"/>
-      <x:c r="L4" s="16" t="str"/>
-      <x:c r="M4" s="16" t="str"/>
-      <x:c r="N4" s="2" t="str"/>
-      <x:c r="O4" s="2" t="str">
+      <x:c r="J4" s="81"/>
+      <x:c r="K4" s="81"/>
+      <x:c r="L4" s="81"/>
+      <x:c r="M4" s="81"/>
+      <x:c r="N4" s="81"/>
+      <x:c r="O4" s="81"/>
+      <x:c r="P4" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P4" s="2" t="str">
+      <x:c r="Q4" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q4" s="14" t="str">
+      <x:c r="R4" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R4" s="17" t="str">
-        <x:v>Ordered regional identity operator bands IMEI attach burst and TLS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="2" t="str">
+      <x:c r="S4" s="81" t="str">
+        <x:v>Verify ordered BG95-M3 marking and firmware identity at incoming; operator SIM attach burst and TLS remain assembled-station EVT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="81" t="str">
         <x:v>RFQ-004</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="str">
+      <x:c r="B5" s="81" t="str">
+        <x:v>U9</x:v>
+      </x:c>
+      <x:c r="C5" s="81" t="str">
         <x:v>GNSS</x:v>
       </x:c>
-      <x:c r="C5" s="2" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>u-blox</x:v>
       </x:c>
-      <x:c r="D5" s="14" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>MAX-M10S-00B</x:v>
       </x:c>
-      <x:c r="E5" s="16" t="n">
+      <x:c r="F5" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F5" s="16" t="n">
+      <x:c r="G5" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G5" s="16" t="n">
+      <x:c r="H5" s="81" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H5" s="2" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Authorized distributor</x:v>
       </x:c>
-      <x:c r="I5" s="2" t="str"/>
-      <x:c r="J5" s="2" t="str"/>
-      <x:c r="K5" s="2" t="str"/>
-      <x:c r="L5" s="16" t="str"/>
-      <x:c r="M5" s="16" t="str"/>
-      <x:c r="N5" s="2" t="str"/>
-      <x:c r="O5" s="2" t="str">
+      <x:c r="J5" s="81"/>
+      <x:c r="K5" s="81"/>
+      <x:c r="L5" s="81"/>
+      <x:c r="M5" s="81"/>
+      <x:c r="N5" s="81"/>
+      <x:c r="O5" s="81"/>
+      <x:c r="P5" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P5" s="2" t="str">
+      <x:c r="Q5" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q5" s="14" t="str">
+      <x:c r="R5" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R5" s="17" t="str">
+      <x:c r="S5" s="81" t="str">
         <x:v>Fix sensitivity PPS and antenna interface</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="2" t="str">
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="81" t="str">
         <x:v>RFQ-005</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="str">
+      <x:c r="B6" s="81" t="str">
+        <x:v>U10</x:v>
+      </x:c>
+      <x:c r="C6" s="81" t="str">
         <x:v>LoRa</x:v>
       </x:c>
-      <x:c r="C6" s="2" t="str">
+      <x:c r="D6" s="81" t="str">
         <x:v>Ebyte</x:v>
       </x:c>
-      <x:c r="D6" s="14" t="str">
+      <x:c r="E6" s="81" t="str">
         <x:v>E22-900M22S</x:v>
       </x:c>
-      <x:c r="E6" s="16" t="n">
+      <x:c r="F6" s="81" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F6" s="16" t="n">
+      <x:c r="G6" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G6" s="16" t="n">
+      <x:c r="H6" s="81" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="H6" s="2" t="str">
+      <x:c r="I6" s="81" t="str">
         <x:v>Ebyte official or authorized</x:v>
       </x:c>
-      <x:c r="I6" s="2" t="str"/>
-      <x:c r="J6" s="2" t="str"/>
-      <x:c r="K6" s="2" t="str"/>
-      <x:c r="L6" s="16" t="str"/>
-      <x:c r="M6" s="16" t="str"/>
-      <x:c r="N6" s="2" t="str"/>
-      <x:c r="O6" s="2" t="str">
+      <x:c r="J6" s="81"/>
+      <x:c r="K6" s="81"/>
+      <x:c r="L6" s="81"/>
+      <x:c r="M6" s="81"/>
+      <x:c r="N6" s="81"/>
+      <x:c r="O6" s="81"/>
+      <x:c r="P6" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P6" s="2" t="str">
+      <x:c r="Q6" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q6" s="14" t="str">
+      <x:c r="R6" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R6" s="17" t="str">
+      <x:c r="S6" s="81" t="str">
         <x:v>Quote and COC must state 20x14 22-pad castellated-ANT option with no module IPEX fitted; conducted RF RU868 windows 864-865 and 868.7-869.2 MHz plus sleep current</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="2" t="str">
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="81" t="str">
         <x:v>RFQ-006</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="str">
+      <x:c r="B7" s="81" t="str">
+        <x:v>U11</x:v>
+      </x:c>
+      <x:c r="C7" s="81" t="str">
         <x:v>BLE</x:v>
       </x:c>
-      <x:c r="C7" s="2" t="str">
+      <x:c r="D7" s="81" t="str">
         <x:v>Raytac</x:v>
       </x:c>
-      <x:c r="D7" s="14" t="str">
+      <x:c r="E7" s="81" t="str">
         <x:v>MDBT50Q-P1MV2</x:v>
       </x:c>
-      <x:c r="E7" s="16" t="n">
+      <x:c r="F7" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F7" s="16" t="n">
+      <x:c r="G7" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G7" s="16" t="n">
+      <x:c r="H7" s="81" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H7" s="2" t="str">
+      <x:c r="I7" s="81" t="str">
         <x:v>Raytac authorized or traceable distributor</x:v>
       </x:c>
-      <x:c r="I7" s="2" t="str"/>
-      <x:c r="J7" s="2" t="str"/>
-      <x:c r="K7" s="2" t="str"/>
-      <x:c r="L7" s="16" t="str"/>
-      <x:c r="M7" s="16" t="str"/>
-      <x:c r="N7" s="2" t="str"/>
-      <x:c r="O7" s="2" t="str">
+      <x:c r="J7" s="81"/>
+      <x:c r="K7" s="81"/>
+      <x:c r="L7" s="81"/>
+      <x:c r="M7" s="81"/>
+      <x:c r="N7" s="81"/>
+      <x:c r="O7" s="81"/>
+      <x:c r="P7" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P7" s="2" t="str">
+      <x:c r="Q7" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q7" s="14" t="str">
+      <x:c r="R7" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R7" s="17" t="str">
+      <x:c r="S7" s="81" t="str">
         <x:v>Exact module suffix integrated-antenna keepout BLE pairing OTA current and RF range</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="2" t="str">
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="81" t="str">
         <x:v>RFQ-007</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="str">
+      <x:c r="B8" s="81" t="str">
+        <x:v>U2</x:v>
+      </x:c>
+      <x:c r="C8" s="81" t="str">
         <x:v>QSPI NOR</x:v>
       </x:c>
-      <x:c r="C8" s="2" t="str">
+      <x:c r="D8" s="81" t="str">
         <x:v>Winbond</x:v>
       </x:c>
-      <x:c r="D8" s="14" t="str">
+      <x:c r="E8" s="81" t="str">
         <x:v>W25Q512JVFIQ</x:v>
       </x:c>
-      <x:c r="E8" s="16" t="n">
+      <x:c r="F8" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F8" s="16" t="n">
+      <x:c r="G8" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G8" s="16" t="n">
+      <x:c r="H8" s="81" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H8" s="2" t="str">
+      <x:c r="I8" s="81" t="str">
         <x:v>Authorized or traceable tier-1</x:v>
       </x:c>
-      <x:c r="I8" s="2" t="str"/>
-      <x:c r="J8" s="2" t="str"/>
-      <x:c r="K8" s="2" t="str"/>
-      <x:c r="L8" s="16" t="str"/>
-      <x:c r="M8" s="16" t="str"/>
-      <x:c r="N8" s="2" t="str"/>
-      <x:c r="O8" s="2" t="str">
+      <x:c r="J8" s="81"/>
+      <x:c r="K8" s="81"/>
+      <x:c r="L8" s="81"/>
+      <x:c r="M8" s="81"/>
+      <x:c r="N8" s="81"/>
+      <x:c r="O8" s="81"/>
+      <x:c r="P8" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P8" s="2" t="str">
+      <x:c r="Q8" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q8" s="14" t="str">
+      <x:c r="R8" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R8" s="17" t="str">
+      <x:c r="S8" s="81" t="str">
         <x:v>JEDEC ID full read write erase soak</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="2" t="str">
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="81" t="str">
         <x:v>RFQ-008</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="str">
+      <x:c r="B9" s="81" t="str">
+        <x:v>BAT1</x:v>
+      </x:c>
+      <x:c r="C9" s="81" t="str">
         <x:v>Battery</x:v>
       </x:c>
-      <x:c r="C9" s="2" t="str">
+      <x:c r="D9" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D9" s="14" t="str">
+      <x:c r="E9" s="81" t="str">
         <x:v>12.8 V 40-60 Ah LiFePO4 with BMS</x:v>
       </x:c>
-      <x:c r="E9" s="16" t="n">
+      <x:c r="F9" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F9" s="16" t="n">
+      <x:c r="G9" s="81" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G9" s="16" t="n">
+      <x:c r="H9" s="81" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="H9" s="2" t="str">
+      <x:c r="I9" s="81" t="str">
         <x:v>Cell or pack manufacturer</x:v>
       </x:c>
-      <x:c r="I9" s="2" t="str"/>
-      <x:c r="J9" s="2" t="str"/>
-      <x:c r="K9" s="2" t="str"/>
-      <x:c r="L9" s="16" t="str"/>
-      <x:c r="M9" s="16" t="str"/>
-      <x:c r="N9" s="2" t="str"/>
-      <x:c r="O9" s="2" t="str">
+      <x:c r="J9" s="81"/>
+      <x:c r="K9" s="81"/>
+      <x:c r="L9" s="81"/>
+      <x:c r="M9" s="81"/>
+      <x:c r="N9" s="81"/>
+      <x:c r="O9" s="81"/>
+      <x:c r="P9" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P9" s="2" t="str">
+      <x:c r="Q9" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q9" s="14" t="str">
+      <x:c r="R9" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R9" s="17" t="str">
+      <x:c r="S9" s="81" t="str">
         <x:v>UN38.3 MSDS capacity DCIR thresholds low-temp inhibit</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="2" t="str">
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="81" t="str">
         <x:v>RFQ-009</x:v>
       </x:c>
-      <x:c r="B10" s="2" t="str">
+      <x:c r="B10" s="81" t="str">
+        <x:v>PV1</x:v>
+      </x:c>
+      <x:c r="C10" s="81" t="str">
         <x:v>Solar</x:v>
       </x:c>
-      <x:c r="C10" s="2" t="str">
+      <x:c r="D10" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D10" s="14" t="str">
+      <x:c r="E10" s="81" t="str">
         <x:v>60-80 W outdoor panel</x:v>
       </x:c>
-      <x:c r="E10" s="16" t="n">
+      <x:c r="F10" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F10" s="16" t="n">
+      <x:c r="G10" s="81" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G10" s="16" t="n">
+      <x:c r="H10" s="81" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="H10" s="2" t="str">
+      <x:c r="I10" s="81" t="str">
         <x:v>Panel manufacturer</x:v>
       </x:c>
-      <x:c r="I10" s="2" t="str"/>
-      <x:c r="J10" s="2" t="str"/>
-      <x:c r="K10" s="2" t="str"/>
-      <x:c r="L10" s="16" t="str"/>
-      <x:c r="M10" s="16" t="str"/>
-      <x:c r="N10" s="2" t="str"/>
-      <x:c r="O10" s="2" t="str">
+      <x:c r="J10" s="81"/>
+      <x:c r="K10" s="81"/>
+      <x:c r="L10" s="81"/>
+      <x:c r="M10" s="81"/>
+      <x:c r="N10" s="81"/>
+      <x:c r="O10" s="81"/>
+      <x:c r="P10" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P10" s="2" t="str">
+      <x:c r="Q10" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q10" s="14" t="str">
+      <x:c r="R10" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R10" s="17" t="str">
+      <x:c r="S10" s="81" t="str">
         <x:v>Voc Isc Pmax insulation weathering evidence</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="2" t="str">
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="81" t="str">
         <x:v>RFQ-010</x:v>
       </x:c>
-      <x:c r="B11" s="2" t="str">
+      <x:c r="B11" s="81" t="str">
+        <x:v>MPPT1</x:v>
+      </x:c>
+      <x:c r="C11" s="81" t="str">
         <x:v>MPPT</x:v>
       </x:c>
-      <x:c r="C11" s="2" t="str">
+      <x:c r="D11" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D11" s="14" t="str">
+      <x:c r="E11" s="81" t="str">
         <x:v>10 A LiFePO4 sealed MPPT</x:v>
       </x:c>
-      <x:c r="E11" s="16" t="n">
+      <x:c r="F11" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F11" s="16" t="n">
+      <x:c r="G11" s="81" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G11" s="16" t="n">
+      <x:c r="H11" s="81" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="H11" s="2" t="str">
+      <x:c r="I11" s="81" t="str">
         <x:v>Controller manufacturer</x:v>
       </x:c>
-      <x:c r="I11" s="2" t="str"/>
-      <x:c r="J11" s="2" t="str"/>
-      <x:c r="K11" s="2" t="str"/>
-      <x:c r="L11" s="16" t="str"/>
-      <x:c r="M11" s="16" t="str"/>
-      <x:c r="N11" s="2" t="str"/>
-      <x:c r="O11" s="2" t="str">
+      <x:c r="J11" s="81"/>
+      <x:c r="K11" s="81"/>
+      <x:c r="L11" s="81"/>
+      <x:c r="M11" s="81"/>
+      <x:c r="N11" s="81"/>
+      <x:c r="O11" s="81"/>
+      <x:c r="P11" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P11" s="2" t="str">
+      <x:c r="Q11" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q11" s="14" t="str">
+      <x:c r="R11" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R11" s="17" t="str">
+      <x:c r="S11" s="81" t="str">
         <x:v>Charge profile cold Voc low-temp reverse current quiescent</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="2" t="str">
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" s="81" t="str">
         <x:v>RFQ-011</x:v>
       </x:c>
-      <x:c r="B12" s="2" t="str">
+      <x:c r="B12" s="81" t="str">
+        <x:v>ASM-MAIN</x:v>
+      </x:c>
+      <x:c r="C12" s="81" t="str">
         <x:v>PCBA main</x:v>
       </x:c>
-      <x:c r="C12" s="2" t="str">
+      <x:c r="D12" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D12" s="14" t="str">
+      <x:c r="E12" s="81" t="str">
         <x:v>6-layer assembled main PCB 110x75x1.6 mm</x:v>
       </x:c>
-      <x:c r="E12" s="16" t="n">
+      <x:c r="F12" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F12" s="16" t="n">
+      <x:c r="G12" s="81" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G12" s="16" t="n">
+      <x:c r="H12" s="81" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H12" s="2" t="str">
+      <x:c r="I12" s="81" t="str">
         <x:v>Qualified CM with AOI</x:v>
       </x:c>
-      <x:c r="I12" s="2" t="str"/>
-      <x:c r="J12" s="2" t="str"/>
-      <x:c r="K12" s="2" t="str"/>
-      <x:c r="L12" s="16" t="str"/>
-      <x:c r="M12" s="16" t="str"/>
-      <x:c r="N12" s="2" t="str"/>
-      <x:c r="O12" s="2" t="str">
+      <x:c r="J12" s="81"/>
+      <x:c r="K12" s="81"/>
+      <x:c r="L12" s="81"/>
+      <x:c r="M12" s="81"/>
+      <x:c r="N12" s="81"/>
+      <x:c r="O12" s="81"/>
+      <x:c r="P12" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P12" s="2" t="str">
+      <x:c r="Q12" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q12" s="14" t="str">
+      <x:c r="R12" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R12" s="17" t="str">
+      <x:c r="S12" s="81" t="str">
         <x:v>final stackup and 50 Ohm coupon; DFM stencil traceability test coverage; MAIN-AUTH-011 outline/keepout compliance</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="2" t="str">
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="81" t="str">
         <x:v>RFQ-012</x:v>
       </x:c>
-      <x:c r="B13" s="2" t="str">
+      <x:c r="B13" s="81" t="str">
+        <x:v>ASM-MIC</x:v>
+      </x:c>
+      <x:c r="C13" s="81" t="str">
         <x:v>PCBA mic</x:v>
       </x:c>
-      <x:c r="C13" s="2" t="str">
+      <x:c r="D13" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D13" s="14" t="str">
+      <x:c r="E13" s="81" t="str">
         <x:v>2-layer assembled microphone PCB</x:v>
       </x:c>
-      <x:c r="E13" s="16" t="n">
+      <x:c r="F13" s="81" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="F13" s="16" t="n">
+      <x:c r="G13" s="81" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="G13" s="16" t="n">
+      <x:c r="H13" s="81" t="n">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="H13" s="2" t="str">
+      <x:c r="I13" s="81" t="str">
         <x:v>Qualified CM with AOI</x:v>
       </x:c>
-      <x:c r="I13" s="2" t="str"/>
-      <x:c r="J13" s="2" t="str"/>
-      <x:c r="K13" s="2" t="str"/>
-      <x:c r="L13" s="16" t="str"/>
-      <x:c r="M13" s="16" t="str"/>
-      <x:c r="N13" s="2" t="str"/>
-      <x:c r="O13" s="2" t="str">
+      <x:c r="J13" s="81"/>
+      <x:c r="K13" s="81"/>
+      <x:c r="L13" s="81"/>
+      <x:c r="M13" s="81"/>
+      <x:c r="N13" s="81"/>
+      <x:c r="O13" s="81"/>
+      <x:c r="P13" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P13" s="2" t="str">
+      <x:c r="Q13" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q13" s="14" t="str">
+      <x:c r="R13" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R13" s="17" t="str">
+      <x:c r="S13" s="81" t="str">
         <x:v>Acoustic port contamination and lot control</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="2" t="str">
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="81" t="str">
         <x:v>RFQ-013</x:v>
       </x:c>
-      <x:c r="B14" s="2" t="str">
+      <x:c r="B14" s="81" t="str">
+        <x:v>ASM-PWR</x:v>
+      </x:c>
+      <x:c r="C14" s="81" t="str">
         <x:v>PCBA power</x:v>
       </x:c>
-      <x:c r="C14" s="2" t="str">
+      <x:c r="D14" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D14" s="14" t="str">
+      <x:c r="E14" s="81" t="str">
         <x:v>assembled power PCB stackup pending DIM-003</x:v>
       </x:c>
-      <x:c r="E14" s="16" t="n">
+      <x:c r="F14" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F14" s="16" t="n">
+      <x:c r="G14" s="81" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G14" s="16" t="n">
+      <x:c r="H14" s="81" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H14" s="2" t="str">
+      <x:c r="I14" s="81" t="str">
         <x:v>Qualified CM with thermal process</x:v>
       </x:c>
-      <x:c r="I14" s="2" t="str"/>
-      <x:c r="J14" s="2" t="str"/>
-      <x:c r="K14" s="2" t="str"/>
-      <x:c r="L14" s="16" t="str"/>
-      <x:c r="M14" s="16" t="str"/>
-      <x:c r="N14" s="2" t="str"/>
-      <x:c r="O14" s="2" t="str">
+      <x:c r="J14" s="81"/>
+      <x:c r="K14" s="81"/>
+      <x:c r="L14" s="81"/>
+      <x:c r="M14" s="81"/>
+      <x:c r="N14" s="81"/>
+      <x:c r="O14" s="81"/>
+      <x:c r="P14" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P14" s="2" t="str">
+      <x:c r="Q14" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q14" s="14" t="str">
+      <x:c r="R14" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R14" s="17" t="str">
+      <x:c r="S14" s="81" t="str">
         <x:v>Current thermal copper Kelvin routing and functional test</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2" t="str">
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="81" t="str">
         <x:v>RFQ-014</x:v>
       </x:c>
-      <x:c r="B15" s="2" t="str">
+      <x:c r="B15" s="81" t="str">
+        <x:v>HARNESS</x:v>
+      </x:c>
+      <x:c r="C15" s="81" t="str">
         <x:v>Harness</x:v>
       </x:c>
-      <x:c r="C15" s="2" t="str">
+      <x:c r="D15" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D15" s="14" t="str">
+      <x:c r="E15" s="81" t="str">
         <x:v>Labeled station harness set</x:v>
       </x:c>
-      <x:c r="E15" s="16" t="n">
+      <x:c r="F15" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F15" s="16" t="n">
+      <x:c r="G15" s="81" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G15" s="16" t="n">
+      <x:c r="H15" s="81" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H15" s="2" t="str">
+      <x:c r="I15" s="81" t="str">
         <x:v>Qualified harness factory</x:v>
       </x:c>
-      <x:c r="I15" s="2" t="str"/>
-      <x:c r="J15" s="2" t="str"/>
-      <x:c r="K15" s="2" t="str"/>
-      <x:c r="L15" s="16" t="str"/>
-      <x:c r="M15" s="16" t="str"/>
-      <x:c r="N15" s="2" t="str"/>
-      <x:c r="O15" s="2" t="str">
+      <x:c r="J15" s="81"/>
+      <x:c r="K15" s="81"/>
+      <x:c r="L15" s="81"/>
+      <x:c r="M15" s="81"/>
+      <x:c r="N15" s="81"/>
+      <x:c r="O15" s="81"/>
+      <x:c r="P15" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P15" s="2" t="str">
+      <x:c r="Q15" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q15" s="14" t="str">
+      <x:c r="R15" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R15" s="17" t="str">
+      <x:c r="S15" s="81" t="str">
         <x:v>Crimp tooling pull force exact lengths and 100 percent continuity</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2" t="str">
+    <x:row r="16" ht="54" customHeight="1">
+      <x:c r="A16" s="81" t="str">
         <x:v>RFQ-015</x:v>
       </x:c>
-      <x:c r="B16" s="2" t="str">
+      <x:c r="B16" s="81" t="str">
+        <x:v>U13</x:v>
+      </x:c>
+      <x:c r="C16" s="81" t="str">
         <x:v>SIM switch</x:v>
       </x:c>
-      <x:c r="C16" s="2" t="str">
+      <x:c r="D16" s="81" t="str">
         <x:v>Texas Instruments</x:v>
       </x:c>
-      <x:c r="D16" s="14" t="str">
+      <x:c r="E16" s="81" t="str">
         <x:v>TS3A27518EPWR</x:v>
       </x:c>
-      <x:c r="E16" s="16" t="n">
+      <x:c r="F16" s="81" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F16" s="16" t="n">
+      <x:c r="G16" s="81" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G16" s="16" t="n">
+      <x:c r="H16" s="81" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H16" s="2" t="str">
+      <x:c r="I16" s="81" t="str">
         <x:v>Authorized distributor</x:v>
       </x:c>
-      <x:c r="I16" s="2" t="str"/>
-      <x:c r="J16" s="2" t="str"/>
-      <x:c r="K16" s="2" t="str"/>
-      <x:c r="L16" s="16" t="str"/>
-      <x:c r="M16" s="16" t="str"/>
-      <x:c r="N16" s="2" t="str"/>
-      <x:c r="O16" s="2" t="str">
+      <x:c r="J16" s="81"/>
+      <x:c r="K16" s="81"/>
+      <x:c r="L16" s="81"/>
+      <x:c r="M16" s="81"/>
+      <x:c r="N16" s="81"/>
+      <x:c r="O16" s="81"/>
+      <x:c r="P16" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P16" s="2" t="str">
+      <x:c r="Q16" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q16" s="14" t="str">
+      <x:c r="R16" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R16" s="17" t="str">
+      <x:c r="S16" s="81" t="str">
         <x:v>Supply leakage Ron capacitance ESD and BG95 signal integrity</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="2" t="str">
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" s="81" t="str">
         <x:v>RFQ-016</x:v>
       </x:c>
-      <x:c r="B17" s="2" t="str">
+      <x:c r="B17" s="81" t="str">
+        <x:v>J-SIM1|J-SIM2</x:v>
+      </x:c>
+      <x:c r="C17" s="81" t="str">
         <x:v>SIM connector</x:v>
       </x:c>
-      <x:c r="C17" s="2" t="str">
+      <x:c r="D17" s="81" t="str">
         <x:v>TE Connectivity</x:v>
       </x:c>
-      <x:c r="D17" s="14" t="str">
+      <x:c r="E17" s="81" t="str">
         <x:v>2336582-1</x:v>
       </x:c>
-      <x:c r="E17" s="16" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F17" s="16" t="n">
+      <x:c r="F17" s="81" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G17" s="81" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="G17" s="16" t="n">
+      <x:c r="H17" s="81" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="H17" s="2" t="str">
+      <x:c r="I17" s="81" t="str">
         <x:v>Authorized or traceable TE distributor</x:v>
       </x:c>
-      <x:c r="I17" s="2" t="str"/>
-      <x:c r="J17" s="2" t="str"/>
-      <x:c r="K17" s="2" t="str"/>
-      <x:c r="L17" s="16" t="str"/>
-      <x:c r="M17" s="16" t="str"/>
-      <x:c r="N17" s="2" t="str"/>
-      <x:c r="O17" s="2" t="str">
+      <x:c r="J17" s="81"/>
+      <x:c r="K17" s="81"/>
+      <x:c r="L17" s="81"/>
+      <x:c r="M17" s="81"/>
+      <x:c r="N17" s="81"/>
+      <x:c r="O17" s="81"/>
+      <x:c r="P17" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P17" s="2" t="str">
+      <x:c r="Q17" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q17" s="14" t="str">
+      <x:c r="R17" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R17" s="17" t="str">
+      <x:c r="S17" s="81" t="str">
         <x:v>Exact drawing revision mating cycles coplanarity card detect and service access</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2" t="str">
+    <x:row r="18" ht="54" customHeight="1">
+      <x:c r="A18" s="81" t="str">
         <x:v>RFQ-017</x:v>
       </x:c>
-      <x:c r="B18" s="2" t="str">
+      <x:c r="B18" s="81" t="str">
+        <x:v>HSG-VC</x:v>
+      </x:c>
+      <x:c r="C18" s="81" t="str">
         <x:v>Vacuum-cast housing</x:v>
       </x:c>
-      <x:c r="C18" s="2" t="str">
+      <x:c r="D18" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D18" s="14" t="str">
+      <x:c r="E18" s="81" t="str">
         <x:v>Outdoor polyurethane housing set with inserts seals and service cover</x:v>
       </x:c>
-      <x:c r="E18" s="16" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F18" s="16" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G18" s="16" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H18" s="2" t="str">
+      <x:c r="F18" s="81" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G18" s="81" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H18" s="81" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I18" s="81" t="str">
         <x:v>Qualified vacuum casting manufacturer</x:v>
       </x:c>
-      <x:c r="I18" s="2" t="str"/>
-      <x:c r="J18" s="2" t="str"/>
-      <x:c r="K18" s="2" t="str"/>
-      <x:c r="L18" s="16" t="str"/>
-      <x:c r="M18" s="16" t="str"/>
-      <x:c r="N18" s="2" t="str"/>
-      <x:c r="O18" s="2" t="str">
+      <x:c r="J18" s="81"/>
+      <x:c r="K18" s="81"/>
+      <x:c r="L18" s="81"/>
+      <x:c r="M18" s="81"/>
+      <x:c r="N18" s="81"/>
+      <x:c r="O18" s="81"/>
+      <x:c r="P18" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P18" s="2" t="str">
+      <x:c r="Q18" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q18" s="14" t="str">
+      <x:c r="R18" s="81" t="str">
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
-      <x:c r="R18" s="17" t="str">
+      <x:c r="S18" s="81" t="str">
         <x:v>FAI shrink cure material UV finish leak fit acoustic and RF checks for selected EVT lot</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="2" t="str">
+    <x:row r="19" ht="54" customHeight="1">
+      <x:c r="A19" s="81" t="str">
         <x:v>RFQ-018</x:v>
       </x:c>
-      <x:c r="B19" s="2" t="str">
+      <x:c r="B19" s="81" t="str">
+        <x:v>HSG-3D</x:v>
+      </x:c>
+      <x:c r="C19" s="81" t="str">
         <x:v>3D-printed fallback housing</x:v>
       </x:c>
-      <x:c r="C19" s="2" t="str">
+      <x:c r="D19" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D19" s="14" t="str">
+      <x:c r="E19" s="81" t="str">
         <x:v>Outdoor printed housing set with inserts seals and service cover</x:v>
       </x:c>
-      <x:c r="E19" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F19" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H19" s="2" t="str">
+      <x:c r="F19" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="81" t="str">
         <x:v>Qualified print supplier or controlled FlashForge 5M Pro process</x:v>
       </x:c>
-      <x:c r="I19" s="2" t="str"/>
-      <x:c r="J19" s="2" t="str"/>
-      <x:c r="K19" s="2" t="str"/>
-      <x:c r="L19" s="16" t="str"/>
-      <x:c r="M19" s="16" t="str"/>
-      <x:c r="N19" s="2" t="str"/>
-      <x:c r="O19" s="2" t="str">
+      <x:c r="J19" s="81"/>
+      <x:c r="K19" s="81"/>
+      <x:c r="L19" s="81"/>
+      <x:c r="M19" s="81"/>
+      <x:c r="N19" s="81"/>
+      <x:c r="O19" s="81"/>
+      <x:c r="P19" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P19" s="2" t="str">
+      <x:c r="Q19" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="Q19" s="14" t="str">
+      <x:c r="R19" s="81" t="str">
         <x:v>CONDITIONAL_CAPACITY_QUOTE</x:v>
       </x:c>
-      <x:c r="R19" s="17" t="str">
+      <x:c r="S19" s="81" t="str">
         <x:v>Quote capacity for 4 10 and 20; procure only after fallback activation</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2" t="str">
+    <x:row r="20" ht="54" customHeight="1">
+      <x:c r="A20" s="81" t="str">
         <x:v>RFQ-019</x:v>
       </x:c>
-      <x:c r="B20" s="2" t="str">
+      <x:c r="B20" s="81" t="str">
+        <x:v>HSG-IM</x:v>
+      </x:c>
+      <x:c r="C20" s="81" t="str">
         <x:v>Injection-molding DFM</x:v>
       </x:c>
-      <x:c r="C20" s="2" t="str">
+      <x:c r="D20" s="81" t="str">
         <x:v>TBD</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="E20" s="81" t="str">
         <x:v>Independent CAD DFM and tool quotation package</x:v>
       </x:c>
-      <x:c r="E20" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F20" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G20" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H20" s="2" t="str">
+      <x:c r="F20" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="81" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="81" t="str">
         <x:v>Qualified mold manufacturer</x:v>
       </x:c>
-      <x:c r="I20" s="2" t="str"/>
-      <x:c r="J20" s="2" t="str"/>
-      <x:c r="K20" s="2" t="str"/>
-      <x:c r="L20" s="16" t="str"/>
-      <x:c r="M20" s="16" t="str"/>
-      <x:c r="N20" s="2" t="str"/>
-      <x:c r="O20" s="2" t="str">
+      <x:c r="J20" s="81"/>
+      <x:c r="K20" s="81"/>
+      <x:c r="L20" s="81"/>
+      <x:c r="M20" s="81"/>
+      <x:c r="N20" s="81"/>
+      <x:c r="O20" s="81"/>
+      <x:c r="P20" s="81" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="P20" s="2" t="str">
+      <x:c r="Q20" s="81" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="Q20" s="14" t="str">
+      <x:c r="R20" s="81" t="str">
         <x:v>SOURCE_DATA_AND_DFM_ONLY</x:v>
       </x:c>
-      <x:c r="R20" s="17" t="str">
+      <x:c r="S20" s="81" t="str">
         <x:v>Review tool concept material draft wall ribs bosses parting ejector shrink and expected tooling lead time; no tooling authorization</x:v>
       </x:c>
     </x:row>
@@ -37509,7 +37592,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaaa898262eb48e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e30c3eb350a4e03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware(bom): refresh antenna RFQ workbook
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R92a04400071047ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R570a8e38c19c40ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R87137cd7919b4b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R632e2102b1134eec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rceec7e5e847f4c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R568f8efb297e453c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R4e450638f4d046c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rd79eec39081f4621"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="13">
     <x:font>
@@ -326,7 +327,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="87">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -497,6 +498,17 @@
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -652,7 +664,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RfqTable" displayName="RfqTable" ref="A1:S20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RfqTable" displayName="RfqTable" ref="A1:S23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="RFQ_ID"/>
     <x:tableColumn id="2" name="BOM_Item_IDs"/>
@@ -1007,7 +1019,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>ba7a886ccb56</x:v>
+        <x:v>5f1332d46691</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10510,7 +10522,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85bf73224a0e4c40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6834f407124aa9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36604,7 +36616,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b4af2bb92324d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7eaab082a814d85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36709,13 +36721,13 @@
       <x:c r="E2" s="81" t="str">
         <x:v>STM32U585VIT6Q</x:v>
       </x:c>
-      <x:c r="F2" s="81" t="n">
+      <x:c r="F2" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" s="81" t="n">
+      <x:c r="G2" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H2" s="81" t="n">
+      <x:c r="H2" s="82" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I2" s="81" t="str">
@@ -36756,13 +36768,13 @@
       <x:c r="E3" s="81" t="str">
         <x:v>MMICT5838-00-012 same lot</x:v>
       </x:c>
-      <x:c r="F3" s="81" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G3" s="81" t="n">
+      <x:c r="F3" s="82" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G3" s="82" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="H3" s="81" t="n">
+      <x:c r="H3" s="82" t="n">
         <x:v>96</x:v>
       </x:c>
       <x:c r="I3" s="81" t="str">
@@ -36803,13 +36815,13 @@
       <x:c r="E4" s="81" t="str">
         <x:v>BG95-M3 marking and firmware identity</x:v>
       </x:c>
-      <x:c r="F4" s="81" t="n">
+      <x:c r="F4" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G4" s="81" t="n">
+      <x:c r="G4" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H4" s="81" t="n">
+      <x:c r="H4" s="82" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I4" s="81" t="str">
@@ -36850,13 +36862,13 @@
       <x:c r="E5" s="81" t="str">
         <x:v>MAX-M10S-00B</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="n">
+      <x:c r="F5" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="n">
+      <x:c r="G5" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="n">
+      <x:c r="H5" s="82" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I5" s="81" t="str">
@@ -36897,13 +36909,13 @@
       <x:c r="E6" s="81" t="str">
         <x:v>E22-900M22S</x:v>
       </x:c>
-      <x:c r="F6" s="81" t="n">
+      <x:c r="F6" s="82" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G6" s="81" t="n">
+      <x:c r="G6" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H6" s="81" t="n">
+      <x:c r="H6" s="82" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="I6" s="81" t="str">
@@ -36944,13 +36956,13 @@
       <x:c r="E7" s="81" t="str">
         <x:v>MDBT50Q-P1MV2</x:v>
       </x:c>
-      <x:c r="F7" s="81" t="n">
+      <x:c r="F7" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G7" s="81" t="n">
+      <x:c r="G7" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H7" s="81" t="n">
+      <x:c r="H7" s="82" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I7" s="81" t="str">
@@ -36991,13 +37003,13 @@
       <x:c r="E8" s="81" t="str">
         <x:v>W25Q512JVFIQ</x:v>
       </x:c>
-      <x:c r="F8" s="81" t="n">
+      <x:c r="F8" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G8" s="81" t="n">
+      <x:c r="G8" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H8" s="81" t="n">
+      <x:c r="H8" s="82" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I8" s="81" t="str">
@@ -37038,13 +37050,13 @@
       <x:c r="E9" s="81" t="str">
         <x:v>12.8 V 40-60 Ah LiFePO4 with BMS</x:v>
       </x:c>
-      <x:c r="F9" s="81" t="n">
+      <x:c r="F9" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G9" s="81" t="n">
+      <x:c r="G9" s="82" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H9" s="81" t="n">
+      <x:c r="H9" s="82" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I9" s="81" t="str">
@@ -37085,13 +37097,13 @@
       <x:c r="E10" s="81" t="str">
         <x:v>60-80 W outdoor panel</x:v>
       </x:c>
-      <x:c r="F10" s="81" t="n">
+      <x:c r="F10" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G10" s="81" t="n">
+      <x:c r="G10" s="82" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H10" s="81" t="n">
+      <x:c r="H10" s="82" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I10" s="81" t="str">
@@ -37132,13 +37144,13 @@
       <x:c r="E11" s="81" t="str">
         <x:v>10 A LiFePO4 sealed MPPT</x:v>
       </x:c>
-      <x:c r="F11" s="81" t="n">
+      <x:c r="F11" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G11" s="81" t="n">
+      <x:c r="G11" s="82" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H11" s="81" t="n">
+      <x:c r="H11" s="82" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I11" s="81" t="str">
@@ -37179,13 +37191,13 @@
       <x:c r="E12" s="81" t="str">
         <x:v>6-layer assembled main PCB 110x75x1.6 mm</x:v>
       </x:c>
-      <x:c r="F12" s="81" t="n">
+      <x:c r="F12" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G12" s="81" t="n">
+      <x:c r="G12" s="82" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H12" s="81" t="n">
+      <x:c r="H12" s="82" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I12" s="81" t="str">
@@ -37226,13 +37238,13 @@
       <x:c r="E13" s="81" t="str">
         <x:v>2-layer assembled microphone PCB</x:v>
       </x:c>
-      <x:c r="F13" s="81" t="n">
+      <x:c r="F13" s="82" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="G13" s="81" t="n">
+      <x:c r="G13" s="82" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="H13" s="81" t="n">
+      <x:c r="H13" s="82" t="n">
         <x:v>88</x:v>
       </x:c>
       <x:c r="I13" s="81" t="str">
@@ -37273,13 +37285,13 @@
       <x:c r="E14" s="81" t="str">
         <x:v>assembled power PCB stackup pending DIM-003</x:v>
       </x:c>
-      <x:c r="F14" s="81" t="n">
+      <x:c r="F14" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G14" s="81" t="n">
+      <x:c r="G14" s="82" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H14" s="81" t="n">
+      <x:c r="H14" s="82" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I14" s="81" t="str">
@@ -37320,13 +37332,13 @@
       <x:c r="E15" s="81" t="str">
         <x:v>Labeled station harness set</x:v>
       </x:c>
-      <x:c r="F15" s="81" t="n">
+      <x:c r="F15" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G15" s="81" t="n">
+      <x:c r="G15" s="82" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H15" s="81" t="n">
+      <x:c r="H15" s="82" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I15" s="81" t="str">
@@ -37367,13 +37379,13 @@
       <x:c r="E16" s="81" t="str">
         <x:v>TS3A27518EPWR</x:v>
       </x:c>
-      <x:c r="F16" s="81" t="n">
+      <x:c r="F16" s="82" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G16" s="81" t="n">
+      <x:c r="G16" s="82" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H16" s="81" t="n">
+      <x:c r="H16" s="82" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I16" s="81" t="str">
@@ -37414,13 +37426,13 @@
       <x:c r="E17" s="81" t="str">
         <x:v>2336582-1</x:v>
       </x:c>
-      <x:c r="F17" s="81" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G17" s="81" t="n">
+      <x:c r="F17" s="82" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G17" s="82" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="H17" s="81" t="n">
+      <x:c r="H17" s="82" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="I17" s="81" t="str">
@@ -37461,13 +37473,13 @@
       <x:c r="E18" s="81" t="str">
         <x:v>Outdoor polyurethane housing set with inserts seals and service cover</x:v>
       </x:c>
-      <x:c r="F18" s="81" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G18" s="81" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H18" s="81" t="n">
+      <x:c r="F18" s="82" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G18" s="82" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H18" s="82" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="I18" s="81" t="str">
@@ -37508,13 +37520,13 @@
       <x:c r="E19" s="81" t="str">
         <x:v>Outdoor printed housing set with inserts seals and service cover</x:v>
       </x:c>
-      <x:c r="F19" s="81" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="81" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H19" s="81" t="n">
+      <x:c r="F19" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="82" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="81" t="str">
@@ -37555,13 +37567,13 @@
       <x:c r="E20" s="81" t="str">
         <x:v>Independent CAD DFM and tool quotation package</x:v>
       </x:c>
-      <x:c r="F20" s="81" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G20" s="81" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H20" s="81" t="n">
+      <x:c r="F20" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="82" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I20" s="81" t="str">
@@ -37586,13 +37598,154 @@
         <x:v>Review tool concept material draft wall ribs bosses parting ejector shrink and expected tooling lead time; no tooling authorization</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A21" s="85" t="str">
+        <x:v>RFQ-020</x:v>
+      </x:c>
+      <x:c r="B21" s="85" t="str">
+        <x:v>ANT-CELL</x:v>
+      </x:c>
+      <x:c r="C21" s="85" t="str">
+        <x:v>Cellular antenna</x:v>
+      </x:c>
+      <x:c r="D21" s="85" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E21" s="85" t="str">
+        <x:v>Outdoor cellular antenna with exact coax and U.FL plug</x:v>
+      </x:c>
+      <x:c r="F21" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G21" s="86" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H21" s="86" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I21" s="85" t="str">
+        <x:v>Antenna manufacturer or authorized distributor</x:v>
+      </x:c>
+      <x:c r="J21" s="85"/>
+      <x:c r="K21" s="85"/>
+      <x:c r="L21" s="85"/>
+      <x:c r="M21" s="85"/>
+      <x:c r="N21" s="85"/>
+      <x:c r="O21" s="85"/>
+      <x:c r="P21" s="85" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q21" s="85" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R21" s="85" t="str">
+        <x:v>RFQ_REQUIRED</x:v>
+      </x:c>
+      <x:c r="S21" s="85" t="str">
+        <x:v>Freeze exact antenna and cable assembly MPN; cover every enabled BG95-M3 deployment band; cable assembly rated at least -40..85 C; provide S11 gain efficiency cable-loss IP evidence and installed-enclosure VSWR/coexistence sample</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A22" s="85" t="str">
+        <x:v>RFQ-021</x:v>
+      </x:c>
+      <x:c r="B22" s="85" t="str">
+        <x:v>ANT-GNSS</x:v>
+      </x:c>
+      <x:c r="C22" s="85" t="str">
+        <x:v>Active GNSS antenna</x:v>
+      </x:c>
+      <x:c r="D22" s="85" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E22" s="85" t="str">
+        <x:v>Outdoor active GNSS L1 antenna with exact coax and U.FL plug</x:v>
+      </x:c>
+      <x:c r="F22" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G22" s="86" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H22" s="86" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I22" s="85" t="str">
+        <x:v>Antenna manufacturer or authorized distributor</x:v>
+      </x:c>
+      <x:c r="J22" s="85"/>
+      <x:c r="K22" s="85"/>
+      <x:c r="L22" s="85"/>
+      <x:c r="M22" s="85"/>
+      <x:c r="N22" s="85"/>
+      <x:c r="O22" s="85"/>
+      <x:c r="P22" s="85" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q22" s="85" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R22" s="85" t="str">
+        <x:v>RFQ_REQUIRED</x:v>
+      </x:c>
+      <x:c r="S22" s="85" t="str">
+        <x:v>Freeze exact antenna and cable assembly MPN; cover 1559.05-1605.66 MHz; operate from 3.3 V at no more than 50 mA; cable assembly rated at least -40..85 C; provide gain noise-figure S11 cable-loss IP evidence and receiver/coexistence sample</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A23" s="85" t="str">
+        <x:v>RFQ-022</x:v>
+      </x:c>
+      <x:c r="B23" s="85" t="str">
+        <x:v>ANT-LORA</x:v>
+      </x:c>
+      <x:c r="C23" s="85" t="str">
+        <x:v>RU868 antenna</x:v>
+      </x:c>
+      <x:c r="D23" s="85" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E23" s="85" t="str">
+        <x:v>Outdoor 868 MHz antenna with exact coax and U.FL plug</x:v>
+      </x:c>
+      <x:c r="F23" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G23" s="86" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H23" s="86" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I23" s="85" t="str">
+        <x:v>Antenna manufacturer or authorized distributor</x:v>
+      </x:c>
+      <x:c r="J23" s="85"/>
+      <x:c r="K23" s="85"/>
+      <x:c r="L23" s="85"/>
+      <x:c r="M23" s="85"/>
+      <x:c r="N23" s="85"/>
+      <x:c r="O23" s="85"/>
+      <x:c r="P23" s="85" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q23" s="85" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R23" s="85" t="str">
+        <x:v>RFQ_REQUIRED</x:v>
+      </x:c>
+      <x:c r="S23" s="85" t="str">
+        <x:v>Freeze exact antenna and cable assembly MPN; cover RU868 windows 864-865 and 868.7-869.2 MHz; cable assembly rated at least -40..85 C; provide S11 gain cable-loss IP evidence installed-enclosure VSWR and conducted/radiated regulatory sample</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="Q2:Q20">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="RFQ_REQUIRED"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e30c3eb350a4e03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a727713148b4049"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware(bom): refresh bare PCB RFQ workbook
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rceec7e5e847f4c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R568f8efb297e453c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R4e450638f4d046c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rd79eec39081f4621"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4d1eed57da2d4965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rf6e23e4ca31b4129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R5c3575c6d80e475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R45d181f0cd54431d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -664,7 +664,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RfqTable" displayName="RfqTable" ref="A1:S23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RfqTable" displayName="RfqTable" ref="A1:S26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="RFQ_ID"/>
     <x:tableColumn id="2" name="BOM_Item_IDs"/>
@@ -1019,7 +1019,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>5f1332d46691</x:v>
+        <x:v>0d19cc829ef7</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10522,7 +10522,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6834f407124aa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6dc257fd1864a15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36616,7 +36616,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7eaab082a814d85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccd08a38623648dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37739,13 +37739,154 @@
         <x:v>Freeze exact antenna and cable assembly MPN; cover RU868 windows 864-865 and 868.7-869.2 MHz; cable assembly rated at least -40..85 C; provide S11 gain cable-loss IP evidence installed-enclosure VSWR and conducted/radiated regulatory sample</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A24" s="81" t="str">
+        <x:v>RFQ-023</x:v>
+      </x:c>
+      <x:c r="B24" s="81" t="str">
+        <x:v>PCB-MAIN</x:v>
+      </x:c>
+      <x:c r="C24" s="81" t="str">
+        <x:v>Bare PCB main</x:v>
+      </x:c>
+      <x:c r="D24" s="81" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E24" s="81" t="str">
+        <x:v>Released PCB-MAIN fabrication package Rev.A</x:v>
+      </x:c>
+      <x:c r="F24" s="82" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G24" s="82" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H24" s="82" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="I24" s="81" t="str">
+        <x:v>Two independent qualified PCB fabricators</x:v>
+      </x:c>
+      <x:c r="J24" s="81"/>
+      <x:c r="K24" s="81"/>
+      <x:c r="L24" s="81"/>
+      <x:c r="M24" s="81"/>
+      <x:c r="N24" s="81"/>
+      <x:c r="O24" s="81"/>
+      <x:c r="P24" s="81" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q24" s="81" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R24" s="81" t="str">
+        <x:v>RFQ_REQUIRED</x:v>
+      </x:c>
+      <x:c r="S24" s="81" t="str">
+        <x:v>Quote and build only from released Gerber drill IPC-356 fabrication drawing and controlled six-layer stackup; preserve the 110 x 75 x 1.60 mm outline from MAIN-AUTH-011; require factory-approved impedance coupon material Tg finish copper weights tolerances net test DFM panelization and lot traceability; no fabrication while routing Review B DRC CAM or DFM is open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A25" s="81" t="str">
+        <x:v>RFQ-024</x:v>
+      </x:c>
+      <x:c r="B25" s="81" t="str">
+        <x:v>PCB-MIC</x:v>
+      </x:c>
+      <x:c r="C25" s="81" t="str">
+        <x:v>Bare PCB microphone</x:v>
+      </x:c>
+      <x:c r="D25" s="81" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E25" s="81" t="str">
+        <x:v>Released PCB-MIC Rev.A 2-layer FR-4 24 x 22 x 1.0 mm ENIG</x:v>
+      </x:c>
+      <x:c r="F25" s="82" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G25" s="82" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H25" s="82" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I25" s="81" t="str">
+        <x:v>Two independent qualified PCB fabricators</x:v>
+      </x:c>
+      <x:c r="J25" s="81"/>
+      <x:c r="K25" s="81"/>
+      <x:c r="L25" s="81"/>
+      <x:c r="M25" s="81"/>
+      <x:c r="N25" s="81"/>
+      <x:c r="O25" s="81"/>
+      <x:c r="P25" s="81" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q25" s="81" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R25" s="81" t="str">
+        <x:v>RFQ_REQUIRED</x:v>
+      </x:c>
+      <x:c r="S25" s="81" t="str">
+        <x:v>Quote and build only from the released Gerber drill IPC-356 and fabrication drawing; preserve the frozen outline mounting holes acoustic opening thickness layer count and ENIG finish; require material Tg copper weights tolerances 100 percent net test panelization/depanel plan DFM and lot traceability; protect the acoustic datum and close Review A Review B and fabricator DFM before manufacture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A26" s="81" t="str">
+        <x:v>RFQ-025</x:v>
+      </x:c>
+      <x:c r="B26" s="81" t="str">
+        <x:v>PCB-PWR</x:v>
+      </x:c>
+      <x:c r="C26" s="81" t="str">
+        <x:v>Bare PCB power</x:v>
+      </x:c>
+      <x:c r="D26" s="81" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E26" s="81" t="str">
+        <x:v>Released PCB-PWR fabrication package after DIM-003 and electrical review</x:v>
+      </x:c>
+      <x:c r="F26" s="82" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G26" s="82" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H26" s="82" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="I26" s="81" t="str">
+        <x:v>Two independent qualified PCB fabricators</x:v>
+      </x:c>
+      <x:c r="J26" s="81"/>
+      <x:c r="K26" s="81"/>
+      <x:c r="L26" s="81"/>
+      <x:c r="M26" s="81"/>
+      <x:c r="N26" s="81"/>
+      <x:c r="O26" s="81"/>
+      <x:c r="P26" s="81" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q26" s="81" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R26" s="81" t="str">
+        <x:v>RFQ_REQUIRED</x:v>
+      </x:c>
+      <x:c r="S26" s="81" t="str">
+        <x:v>Prequote variants must be marked provisional and are not build authorization; final quotation and fabrication await DIM-003 plus released outline mounting stackup copper weight routing and CAM; require material Tg finish copper and plating tolerances current and Kelvin review 100 percent net test DFM panelization and lot traceability; no fabrication from the present placement candidate</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="Q2:Q20">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="RFQ_REQUIRED"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a727713148b4049"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dba3c53a65248ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware(bom): mark selected EVT-20 scenario
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4d1eed57da2d4965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rf6e23e4ca31b4129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R5c3575c6d80e475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R45d181f0cd54431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfcb0554882f64356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R36077518d96a4cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rc57c6b321577444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R1465d81c0bb84679"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -89,8 +89,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFC62828"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -117,8 +123,23 @@
         <x:fgColor rgb="FFFFF7ED"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE9E7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="23">
+  <x:borders count="26">
     <x:border/>
     <x:border>
       <x:right style="thin">
@@ -323,11 +344,41 @@
         <x:color rgb="FFFED7AA"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="87">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -508,6 +559,44 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -982,28 +1071,48 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="33" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="n">
+      <x:c r="A8" s="93" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B8" s="94" t="n">
         <x:f>SUMIF('Engineering BOM'!$A$2:$A$294,"ASM-MAIN",'Engineering BOM'!$P$2:$P$294)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C8" s="34" t="n">
+      <x:c r="C8" s="94" t="n">
         <x:f>SUMIF('Engineering BOM'!$A$2:$A$294,"ASM-PWR",'Engineering BOM'!$P$2:$P$294)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D8" s="34" t="n">
+      <x:c r="D8" s="94" t="n">
         <x:f>SUMIF('Engineering BOM'!$A$2:$A$294,"ASM-MIC",'Engineering BOM'!$P$2:$P$294)</x:f>
         <x:v>80</x:v>
       </x:c>
-      <x:c r="E8" s="34" t="n">
+      <x:c r="E8" s="94" t="n">
         <x:f>SUMIF('Engineering BOM'!$A$2:$A$294,"MK1",'Engineering BOM'!$P$2:$P$294)</x:f>
         <x:v>80</x:v>
       </x:c>
-      <x:c r="F8" s="35" t="n">
+      <x:c r="F8" s="95" t="n">
         <x:f>SUMIF('Engineering BOM'!$A$2:$A$294,"HSG-VC",'Engineering BOM'!$P$2:$P$294)</x:f>
         <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="20" customHeight="1">
+      <x:c r="A9" s="101" t="str">
+        <x:v>Selected scenario</x:v>
+      </x:c>
+      <x:c r="B9" s="102" t="str">
+        <x:v>EVT-20</x:v>
+      </x:c>
+      <x:c r="C9" s="102" t="str">
+        <x:v>20 stations</x:v>
+      </x:c>
+      <x:c r="D9" s="102" t="str">
+        <x:v>DIO-EVT-001..020</x:v>
+      </x:c>
+      <x:c r="E9" s="102" t="str">
+        <x:v>Purchase gate</x:v>
+      </x:c>
+      <x:c r="F9" s="106" t="str">
+        <x:v>BLOCKED</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1019,7 +1128,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>0d19cc829ef7</x:v>
+        <x:v>037e918f3559</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10522,7 +10631,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6dc257fd1864a15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R318c2050de674631"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36616,7 +36725,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccd08a38623648dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc001b1e382344931"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37886,7 +37995,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dba3c53a65248ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb91b360ac65b4194"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware: remediate review layer and harness gaps
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfcb0554882f64356"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R36077518d96a4cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rc57c6b321577444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R1465d81c0bb84679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf811649c15a44016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rcd92b790c1fb4528"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R3a137e3ceec542f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R9d9da1f04dde4f8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1731,7 +1731,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="H7" s="2" t="str">
-        <x:v>2-layer 2 oz candidate</x:v>
+        <x:v>4-layer PCBA; outer 2 oz target; inner 1 oz target; final stackup pending DFM</x:v>
       </x:c>
       <x:c r="I7" s="2" t="str"/>
       <x:c r="J7" s="2" t="str">
@@ -2406,7 +2406,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="H16" s="2" t="str">
-        <x:v>2-layer 2 oz candidate</x:v>
+        <x:v>4-layer FR-4; outer 2 oz target; inner 1 oz target; final stackup pending DFM</x:v>
       </x:c>
       <x:c r="I16" s="2" t="str"/>
       <x:c r="J16" s="2" t="str">
@@ -10631,7 +10631,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R318c2050de674631"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd693adc633c14b49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13658,7 +13658,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
-        <x:v>2-layer 2 oz candidate</x:v>
+        <x:v>4-layer PCBA; outer 2 oz target; inner 1 oz target; final stackup pending DFM</x:v>
       </x:c>
       <x:c r="I35" s="16" t="n">
         <x:v>1</x:v>
@@ -13706,7 +13706,7 @@
         <x:v>AOI functional high-current thermal</x:v>
       </x:c>
       <x:c r="X35" s="17" t="str">
-        <x:v>No MPPT function on this board</x:v>
+        <x:v>No MPPT function on this board; layer count frozen but copper weights and construction remain open</x:v>
       </x:c>
       <x:c r="Y35" s="2" t="str"/>
       <x:c r="Z35" s="2" t="str">
@@ -13745,7 +13745,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="H36" s="2" t="str">
-        <x:v>2-layer 2 oz candidate</x:v>
+        <x:v>4-layer FR-4; outer 2 oz target; inner 1 oz target; final stackup pending DFM</x:v>
       </x:c>
       <x:c r="I36" s="16" t="n">
         <x:v>1</x:v>
@@ -13793,7 +13793,7 @@
         <x:v>Copper thickness netlist high-current and Kelvin review</x:v>
       </x:c>
       <x:c r="X36" s="17" t="str">
-        <x:v>Final copper weight by current calculation</x:v>
+        <x:v>Layer count frozen; final copper weights by current and thermal calculation plus fabricator DFM</x:v>
       </x:c>
       <x:c r="Y36" s="2" t="str"/>
       <x:c r="Z36" s="2" t="str">
@@ -36725,7 +36725,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc001b1e382344931"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f608d59bf584d35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37392,7 +37392,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="E14" s="81" t="str">
-        <x:v>assembled power PCB stackup pending DIM-003</x:v>
+        <x:v>assembled 4-layer power PCB; outer 2 oz target; inner 1 oz target; final stackup pending DFM and DIM-003</x:v>
       </x:c>
       <x:c r="F14" s="82" t="n">
         <x:v>5</x:v>
@@ -37956,7 +37956,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="E26" s="81" t="str">
-        <x:v>Released PCB-PWR fabrication package after DIM-003 and electrical review</x:v>
+        <x:v>4-layer FR-4 PCB; outer 2 oz target; inner 1 oz target; final stackup pending DFM and DIM-003</x:v>
       </x:c>
       <x:c r="F26" s="82" t="n">
         <x:v>5</x:v>
@@ -37995,7 +37995,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb91b360ac65b4194"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cd9b9ddf9984eca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware: bind BOM workbook to published baseline
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R22eb0f8d02604271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Re1ce1368ee2c43b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R7b824cecfaf64c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rb278982dbed84983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R90683e3546ab4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rd647729b430340c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R6457300e89d54c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rdf8afa8242b247d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1137,7 +1137,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>cbce3b5b48bb</x:v>
+        <x:v>2dda0727b009</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10790,7 +10790,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref037449ca7b4c21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reae76111e9b945a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37058,7 +37058,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ff2b4be7fdc46f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcff279da2ce4b19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38438,7 +38438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8332c62900c43ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6b69f605bb4b03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware: refresh BOM workbook after F1 ECO
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R90683e3546ab4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rd647729b430340c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R6457300e89d54c6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rdf8afa8242b247d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rffaf73b0f0244cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rde1b0b8a11284f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rf9943804f7f8463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R6d0d725863fd4bce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1137,7 +1137,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>2dda0727b009</x:v>
+        <x:v>3cdaef294481</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1218,7 +1218,7 @@
         <x:v>PWR-TVS-01, PWR-FUSE-01, HSG-VC</x:v>
       </x:c>
       <x:c r="C23" s="73" t="str">
-        <x:v>Apply bounded F1 native value ECO; close 20/20 input-protection tests and housing FAI supplier release</x:v>
+        <x:v>Collect post-ECO F1 ERC/PDF and human hierarchy review; close 20/20 input-protection tests and housing FAI supplier release</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2158,7 +2158,7 @@
         <x:v>BLOCKED_ENGINEERING_SELECTION</x:v>
       </x:c>
       <x:c r="W12" s="14" t="str">
-        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_PENDING</x:v>
+        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PENDING</x:v>
       </x:c>
       <x:c r="X12" s="17" t="str">
         <x:v>Authorized distributor</x:v>
@@ -10790,7 +10790,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reae76111e9b945a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a7f00744e04d26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13769,7 +13769,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U34" s="14" t="str">
-        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_PENDING</x:v>
+        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PENDING</x:v>
       </x:c>
       <x:c r="V34" s="17" t="str">
         <x:v>Authorized distributor</x:v>
@@ -13778,7 +13778,7 @@
         <x:v>Marking continuity and controlled fault clearing</x:v>
       </x:c>
       <x:c r="X34" s="17" t="str">
-        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 8 A nominal; 0.0077 Ohm nominal cold resistance; 20.23 A2s nominal melting I2t; standard 25% continuous derating plus temperature rerating required; blockers: signed native value still 0451005.MRL; repeat ERC/PDF/human hierarchy review after value-only ECO; +70 C derating; inrush; fault energy; 8.5 A connector ceiling; battery-side primary-fuse coordination</x:v>
+        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 8 A nominal; 0.0077 Ohm nominal cold resistance; 20.23 A2s nominal melting I2t; standard 25% continuous derating plus temperature rerating required; blockers: native value-only ECO applied with footprint placement topology and nets retained; repeat ERC/PDF/human hierarchy review; +70 C derating; inrush; fault energy; 8.5 A connector ceiling; battery-side primary-fuse coordination</x:v>
       </x:c>
       <x:c r="Y34" s="2" t="str"/>
       <x:c r="Z34" s="2" t="str">
@@ -37058,7 +37058,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcff279da2ce4b19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab1561fd62084af6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38438,7 +38438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6b69f605bb4b03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b878ca29d874285"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
release: synchronize integration baseline v0.14
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R90683e3546ab4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rd647729b430340c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R6457300e89d54c6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rdf8afa8242b247d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rffaf73b0f0244cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rde1b0b8a11284f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rf9943804f7f8463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R6d0d725863fd4bce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1137,7 +1137,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>2dda0727b009</x:v>
+        <x:v>3cdaef294481</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1218,7 +1218,7 @@
         <x:v>PWR-TVS-01, PWR-FUSE-01, HSG-VC</x:v>
       </x:c>
       <x:c r="C23" s="73" t="str">
-        <x:v>Apply bounded F1 native value ECO; close 20/20 input-protection tests and housing FAI supplier release</x:v>
+        <x:v>Collect post-ECO F1 ERC/PDF and human hierarchy review; close 20/20 input-protection tests and housing FAI supplier release</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2158,7 +2158,7 @@
         <x:v>BLOCKED_ENGINEERING_SELECTION</x:v>
       </x:c>
       <x:c r="W12" s="14" t="str">
-        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_PENDING</x:v>
+        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PENDING</x:v>
       </x:c>
       <x:c r="X12" s="17" t="str">
         <x:v>Authorized distributor</x:v>
@@ -10790,7 +10790,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reae76111e9b945a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a7f00744e04d26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13769,7 +13769,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U34" s="14" t="str">
-        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_PENDING</x:v>
+        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PENDING</x:v>
       </x:c>
       <x:c r="V34" s="17" t="str">
         <x:v>Authorized distributor</x:v>
@@ -13778,7 +13778,7 @@
         <x:v>Marking continuity and controlled fault clearing</x:v>
       </x:c>
       <x:c r="X34" s="17" t="str">
-        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 8 A nominal; 0.0077 Ohm nominal cold resistance; 20.23 A2s nominal melting I2t; standard 25% continuous derating plus temperature rerating required; blockers: signed native value still 0451005.MRL; repeat ERC/PDF/human hierarchy review after value-only ECO; +70 C derating; inrush; fault energy; 8.5 A connector ceiling; battery-side primary-fuse coordination</x:v>
+        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 8 A nominal; 0.0077 Ohm nominal cold resistance; 20.23 A2s nominal melting I2t; standard 25% continuous derating plus temperature rerating required; blockers: native value-only ECO applied with footprint placement topology and nets retained; repeat ERC/PDF/human hierarchy review; +70 C derating; inrush; fault energy; 8.5 A connector ceiling; battery-side primary-fuse coordination</x:v>
       </x:c>
       <x:c r="Y34" s="2" t="str"/>
       <x:c r="Z34" s="2" t="str">
@@ -37058,7 +37058,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcff279da2ce4b19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab1561fd62084af6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38438,7 +38438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6b69f605bb4b03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b878ca29d874285"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware: sync controlled BOM workbook
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rffaf73b0f0244cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rde1b0b8a11284f75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rf9943804f7f8463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R6d0d725863fd4bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd052d8f8ebb041f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Re4707379e5b14104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R5fd65ff31b16400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R2af50861e5834212"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3538,7 +3538,7 @@
         <x:v>PWR-C-CIN-HF</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>C9</x:v>
+        <x:v>C9;C20;C21</x:v>
       </x:c>
       <x:c r="E31" s="2" t="str">
         <x:v>Passive</x:v>
@@ -3562,31 +3562,31 @@
         <x:v>FITTED</x:v>
       </x:c>
       <x:c r="L31" s="16" t="str">
-        <x:v>4</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="M31" s="16" t="str">
         <x:v>40</x:v>
       </x:c>
       <x:c r="N31" s="16" t="str">
-        <x:v>44</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="O31" s="16" t="str">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="P31" s="16" t="str">
         <x:v>40</x:v>
       </x:c>
       <x:c r="Q31" s="16" t="str">
-        <x:v>50</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="R31" s="16" t="str">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="S31" s="16" t="str">
         <x:v>40</x:v>
       </x:c>
       <x:c r="T31" s="16" t="str">
-        <x:v>60</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="U31" s="14" t="str">
         <x:v>FIXED_LOT_MIN</x:v>
@@ -3595,7 +3595,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W31" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_TRANSIENT</x:v>
+        <x:v>CONTROLLED_CANDIDATE_PENDING_MULTIPLE_REVIEWS</x:v>
       </x:c>
       <x:c r="X31" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10790,7 +10790,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a7f00744e04d26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31ed16d21c024a07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13167,7 +13167,7 @@
         <x:v>Load step ripple efficiency thermal and EMI</x:v>
       </x:c>
       <x:c r="X27" s="17" t="str">
-        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 3-36 V input; 4 A; adjustable output set to 3.8 V; low-Iq synchronous buck; blockers: capacitor/feedback verification; 2.7 A+ BG95 burst test; EMI; thermal</x:v>
+        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 3-36 V input; 4 A; TI-verified adjustable mode; 3.8 V nominal; low-Iq synchronous buck; blockers: C11 effective capacitance under bias; C20 local CIN_HF placement; 2.7 A+ BG95 burst; EMI; thermal</x:v>
       </x:c>
       <x:c r="Y27" s="2" t="str"/>
       <x:c r="Z27" s="2" t="str">
@@ -13254,7 +13254,7 @@
         <x:v>Load step ripple efficiency sleep current thermal and EMI</x:v>
       </x:c>
       <x:c r="X28" s="17" t="str">
-        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 3-36 V input; 4 A; output set to 3.3 V; low-Iq synchronous buck; blockers: capacitor verification; load-step; sleep-current; EMI; thermal</x:v>
+        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 3-36 V input; 4 A; TI-verified fixed 3.3 V mode; low-Iq synchronous buck; blockers: C12 effective capacitance under bias; C21 local CIN_HF placement; load-step; sleep-current; EMI; thermal</x:v>
       </x:c>
       <x:c r="Y28" s="2" t="str"/>
       <x:c r="Z28" s="2" t="str">
@@ -35632,7 +35632,7 @@
         <x:v>PCB-PWR</x:v>
       </x:c>
       <x:c r="C281" s="14" t="str">
-        <x:v>C9</x:v>
+        <x:v>C9;C20;C21</x:v>
       </x:c>
       <x:c r="D281" s="2" t="str">
         <x:v>Passive</x:v>
@@ -35650,34 +35650,34 @@
         <x:v>0603</x:v>
       </x:c>
       <x:c r="I281" s="16" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J281" s="16" t="str">
-        <x:v>4</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K281" s="16" t="str">
         <x:v>40</x:v>
       </x:c>
       <x:c r="L281" s="16" t="str">
-        <x:v>44</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="M281" s="16" t="str">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="N281" s="16" t="str">
         <x:v>40</x:v>
       </x:c>
       <x:c r="O281" s="16" t="str">
-        <x:v>50</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="P281" s="16" t="str">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="Q281" s="16" t="str">
         <x:v>40</x:v>
       </x:c>
       <x:c r="R281" s="16" t="str">
-        <x:v>60</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="S281" s="14" t="str">
         <x:v>FIXED_LOT_MIN</x:v>
@@ -35686,7 +35686,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U281" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_TRANSIENT</x:v>
+        <x:v>CONTROLLED_CANDIDATE_PENDING_MULTIPLE_REVIEWS</x:v>
       </x:c>
       <x:c r="V281" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -35695,7 +35695,7 @@
         <x:v>Marking MPN package orientation electrical functional sample</x:v>
       </x:c>
       <x:c r="X281" s="17" t="str">
-        <x:v>Rev.A source PCB_PWR_PASSIVE_AUTHORITY_REV_A.csv; footprint Capacitor_SMD:C_0603_1608Metric; blockers: transient profile and TVS coordination</x:v>
+        <x:v>Rev.A source PCB_PWR_PASSIVE_AUTHORITY_REV_A.csv; footprint Capacitor_SMD:C_0603_1608Metric; blockers: DC bias high-frequency loop placement and EMI review; transient profile and TVS coordination</x:v>
       </x:c>
       <x:c r="Y281" s="2" t="str">
         <x:v>100 nF 50 V X7R</x:v>
@@ -37058,7 +37058,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab1561fd62084af6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5c9257189894c1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38438,7 +38438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b878ca29d874285"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f77bfb10fff4aab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
pcb-pwr: record active hierarchy acceptance
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd052d8f8ebb041f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Re4707379e5b14104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R5fd65ff31b16400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R2af50861e5834212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R37e21196c4714afa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R02fb9af2ecb74b47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R2f6b37a179924dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Refd260fb4d004d33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1218,7 +1218,7 @@
         <x:v>PWR-TVS-01, PWR-FUSE-01, HSG-VC</x:v>
       </x:c>
       <x:c r="C23" s="73" t="str">
-        <x:v>Collect post-ECO F1 ERC/PDF and human hierarchy review; close 20/20 input-protection tests and housing FAI supplier release</x:v>
+        <x:v>Close the remaining 18/20 PCB-PWR input-protection physical tests and housing FAI supplier release</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2158,7 +2158,7 @@
         <x:v>BLOCKED_ENGINEERING_SELECTION</x:v>
       </x:c>
       <x:c r="W12" s="14" t="str">
-        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PENDING</x:v>
+        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PASS_PHYSICAL_QUALIFICATION_PENDING</x:v>
       </x:c>
       <x:c r="X12" s="17" t="str">
         <x:v>Authorized distributor</x:v>
@@ -10790,7 +10790,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31ed16d21c024a07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c8288f1ffeb42d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13769,7 +13769,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U34" s="14" t="str">
-        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PENDING</x:v>
+        <x:v>CANDIDATE_SELECTED_FOR_EVT_QUALIFICATION_NATIVE_VALUE_ECO_APPLIED_REPEAT_EVIDENCE_PASS_PHYSICAL_QUALIFICATION_PENDING</x:v>
       </x:c>
       <x:c r="V34" s="17" t="str">
         <x:v>Authorized distributor</x:v>
@@ -13778,7 +13778,7 @@
         <x:v>Marking continuity and controlled fault clearing</x:v>
       </x:c>
       <x:c r="X34" s="17" t="str">
-        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 8 A nominal; 0.0077 Ohm nominal cold resistance; 20.23 A2s nominal melting I2t; standard 25% continuous derating plus temperature rerating required; blockers: native value-only ECO applied with footprint placement topology and nets retained; repeat ERC/PDF/human hierarchy review; +70 C derating; inrush; fault energy; 8.5 A connector ceiling; battery-side primary-fuse coordination</x:v>
+        <x:v>Rev.A freeze source POWER_COMPONENT_FREEZE_REV_A.csv; 8 A nominal; 0.0077 Ohm nominal cold resistance; 20.23 A2s nominal melting I2t; standard 25% continuous derating plus temperature rerating required; blockers: native value-only ECO applied with footprint placement topology and nets retained; repeat ERC/PDF/human hierarchy review PASS; +70 C derating; inrush; fault energy; 8.5 A connector ceiling; battery-side primary-fuse coordination</x:v>
       </x:c>
       <x:c r="Y34" s="2" t="str"/>
       <x:c r="Z34" s="2" t="str">
@@ -37058,7 +37058,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5c9257189894c1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd8cac279d004b77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38438,7 +38438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f77bfb10fff4aab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R512da55076dd4212"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
bom: audit full PCBA cost tracks
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd1bcfdf207cb415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R53d764f885c74c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rabefd6d16aec418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rf625bd708b554f02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R5b1eb8b480e94e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R31688eb2c4564aef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Ra72304e1d2e743ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R97781bc9bce14d76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R109abf1df9a44598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R40490ce15c4b4faf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1567,7 +1567,7 @@
         <x:v>Source commit</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>689b0c42d0bf</x:v>
+        <x:v>cf9ee11a9491</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -11232,7 +11232,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce318ed0bf464dd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4e4eb0a375747d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37500,7 +37500,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97cf13c809224a46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reca94d4aec864274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38880,7 +38880,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dbd14d5c4ea4af6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R648f00ac36a44654"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46202,7 +46202,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf81f65b9f2a042f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb74e163fcdd04854"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
hardware: accept PCB-PWR EVT mechanical authority
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R31688eb2c4564aef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Ra72304e1d2e743ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R97781bc9bce14d76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R109abf1df9a44598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R40490ce15c4b4faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R58352d42e169410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R5ac2f8986e744106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R7bd15f0b5ac6427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R5b32fd3412eb4a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="Rc4abb065d37a4143"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11232,7 +11232,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4e4eb0a375747d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76f6539921fd4217"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37500,7 +37500,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reca94d4aec864274"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71b3c1d3e9434ca6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38173,7 +38173,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="E14" s="81" t="str">
-        <x:v>assembled 4-layer power PCB; outer 2 oz target; inner 1 oz target; final stackup pending DFM and DIM-003</x:v>
+        <x:v>assembled 4-layer power PCB; EVT DIM-003 90x60x1.6 mm and H1-H4 accepted; outer 2 oz target; inner 1 oz target; final stackup pending DFM</x:v>
       </x:c>
       <x:c r="F14" s="82" t="str">
         <x:v>6</x:v>
@@ -38203,7 +38203,7 @@
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
       <x:c r="S14" s="81" t="str">
-        <x:v>PRIMARY PROCUREMENT TRACK; quote only after final stackup DIM-003 routing DRC CAM DFM and Review B; retain 100 percent AOI and EOL plus current thermal copper Kelvin and fault validation on the selected lot</x:v>
+        <x:v>PRIMARY PROCUREMENT TRACK; quote only after accepted stackup routing DRC CAM DFM serial mechanical revalidation and Review B; retain 100 percent AOI and EOL plus current thermal copper Kelvin and fault validation on the selected lot</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -38250,7 +38250,7 @@
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
       <x:c r="S15" s="81" t="str">
-        <x:v>Return all 16 attributable rows in HARNESS_SUPPLIER_CAPABILITY_RESPONSE_REV_A.csv including site assembly MPN complete-harness temperature wire AVL crimp FAI traceability and quote; no build until DIM-001 DIM-003 DIM-012 and final release; first article is part of the selected lot</x:v>
+        <x:v>Return all 16 attributable rows in HARNESS_SUPPLIER_CAPABILITY_RESPONSE_REV_A.csv including site assembly MPN complete-harness temperature wire AVL crimp FAI traceability and quote; DIM-003 board datums are EVT accepted but no build until DIM-001 DIM-005 DIM-006 DIM-012 final enclosure routes and final release; first article is part of the selected lot</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -38743,7 +38743,7 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="E26" s="81" t="str">
-        <x:v>4-layer FR-4 PCB; outer 2 oz target; inner 1 oz target; final stackup pending DFM and DIM-003</x:v>
+        <x:v>4-layer FR-4 PCB; EVT DIM-003 90x60x1.6 mm and H1-H4 accepted; outer 2 oz target; inner 1 oz target; final stackup pending DFM</x:v>
       </x:c>
       <x:c r="F26" s="82" t="str">
         <x:v>6</x:v>
@@ -38773,7 +38773,7 @@
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
       <x:c r="S26" s="81" t="str">
-        <x:v>ALTERNATIVE QUOTATION TRACK ONLY; do not issue a purchase order together with ASM-PWR; prequote variants must be marked provisional and are not build authorization; final quotation and fabrication await DIM-003 released outline mounting stackup copper routing and CAM; require material finish copper and plating tolerances current and Kelvin review 100 percent net test DFM panelization traceability and selected-lot FAI</x:v>
+        <x:v>ALTERNATIVE QUOTATION TRACK ONLY; do not issue a purchase order together with ASM-PWR; EVT mechanical values are quotation inputs not build authorization; final quotation and fabrication await accepted stackup copper routing CAM serial mechanical revalidation and release; require material finish copper and plating tolerances current and Kelvin review 100 percent net test DFM panelization traceability and selected-lot FAI</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -38880,7 +38880,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R648f00ac36a44654"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52659db785274d61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46202,7 +46202,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb74e163fcdd04854"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0c0f8a011c44450"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
bom: restore PCB-MIC RFQ dimensional contract
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R83ff1aa49dca4c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rcc58e357ab1b4a2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rb3a3bed6a88a48b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Ra6293321b99d488f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R330a7daf7ffe468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2480a0c201ab4b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R34c7a72beeeb44fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="R999d63c6f8e94647"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="Rfa40c956d0404884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="Ra964330f63e04036"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11280,7 +11280,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8f47299aa91492b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c48b1a9f27e455c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37548,7 +37548,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6264c967ae764b08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f5c7a263f3c493f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38744,7 +38744,7 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="E25" s="81" t="str">
-        <x:v>DIO-PCB-MIC-REV-A released 2-layer FR-4 microphone PCB build-to-print scope</x:v>
+        <x:v>DIO-PCB-MIC-REV-A 2-layer FR-4 24 x 22 x 1.0 mm ENIG microphone PCB build-to-print scope</x:v>
       </x:c>
       <x:c r="F25" s="82" t="str">
         <x:v>18</x:v>
@@ -38928,7 +38928,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c75c36fd2047d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c8afa65f8f548a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45878,7 +45878,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f142b030ce4237"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe4fa5e39908440f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile 2x20+1 traceability and current routing state
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6020cf47624847c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Re1daae1abc364711"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Ra41adccc234a49c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R0a5229325084434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="Rd828dbbeedd7402e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program 41" sheetId="6" r:id="R5518869de1434812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1efdf6b8561447e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rd90521b2a91645ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Reea0dd1abd7540ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R3017a3b854c24ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R8340d9c1023249f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program 41" sheetId="6" r:id="R35d0b331236d436b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -180,7 +180,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -295,6 +295,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -607,7 +612,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="225">
+  <x:cellXfs count="228">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1123,6 +1128,15 @@
     <x:xf numFmtId="0" fontId="26" fillId="26" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="27" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11400,7 +11414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75458bde0c7b4ab1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcacf16b3d3744940"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37668,7 +37682,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6915f66a4b0f4b6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f598f39f5a24813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39048,7 +39062,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33de3b44a417409b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a15d8008f6c4ca8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45998,7 +46012,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R540f257b38834e36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8606e9aaabc346f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46035,79 +46049,79 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="224" t="str">
+      <x:c r="A1" s="227" t="str">
         <x:v>Program_Procurement_ID</x:v>
       </x:c>
-      <x:c r="B1" s="224" t="str">
+      <x:c r="B1" s="227" t="str">
         <x:v>Procurement_ID</x:v>
       </x:c>
-      <x:c r="C1" s="224" t="str">
+      <x:c r="C1" s="227" t="str">
         <x:v>Assemblies</x:v>
       </x:c>
-      <x:c r="D1" s="224" t="str">
+      <x:c r="D1" s="227" t="str">
         <x:v>Item_IDs</x:v>
       </x:c>
-      <x:c r="E1" s="224" t="str">
+      <x:c r="E1" s="227" t="str">
         <x:v>Category</x:v>
       </x:c>
-      <x:c r="F1" s="224" t="str">
+      <x:c r="F1" s="227" t="str">
         <x:v>Manufacturer</x:v>
       </x:c>
-      <x:c r="G1" s="224" t="str">
+      <x:c r="G1" s="227" t="str">
         <x:v>MPN</x:v>
       </x:c>
-      <x:c r="H1" s="224" t="str">
+      <x:c r="H1" s="227" t="str">
         <x:v>Package</x:v>
       </x:c>
-      <x:c r="I1" s="224" t="str">
+      <x:c r="I1" s="227" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="J1" s="224" t="str">
+      <x:c r="J1" s="227" t="str">
         <x:v>Variant</x:v>
       </x:c>
-      <x:c r="K1" s="224" t="str">
+      <x:c r="K1" s="227" t="str">
         <x:v>Population</x:v>
       </x:c>
-      <x:c r="L1" s="224" t="str">
+      <x:c r="L1" s="227" t="str">
         <x:v>Qty_per_station</x:v>
       </x:c>
-      <x:c r="M1" s="224" t="str">
+      <x:c r="M1" s="227" t="str">
         <x:v>Production_lots_20</x:v>
       </x:c>
-      <x:c r="N1" s="224" t="str">
+      <x:c r="N1" s="227" t="str">
         <x:v>Bench_stations</x:v>
       </x:c>
-      <x:c r="O1" s="224" t="str">
+      <x:c r="O1" s="227" t="str">
         <x:v>Total_stations</x:v>
       </x:c>
-      <x:c r="P1" s="224" t="str">
+      <x:c r="P1" s="227" t="str">
         <x:v>Base_qty_2x20_plus_1</x:v>
       </x:c>
-      <x:c r="Q1" s="224" t="str">
+      <x:c r="Q1" s="227" t="str">
         <x:v>Spare_qty_two_evt20_lots</x:v>
       </x:c>
-      <x:c r="R1" s="224" t="str">
+      <x:c r="R1" s="227" t="str">
         <x:v>Procure_qty_2x20_plus_1</x:v>
       </x:c>
-      <x:c r="S1" s="224" t="str">
+      <x:c r="S1" s="227" t="str">
         <x:v>Spare_policy</x:v>
       </x:c>
-      <x:c r="T1" s="224" t="str">
+      <x:c r="T1" s="227" t="str">
         <x:v>Procurement_track</x:v>
       </x:c>
-      <x:c r="U1" s="224" t="str">
+      <x:c r="U1" s="227" t="str">
         <x:v>BOM_disposition</x:v>
       </x:c>
-      <x:c r="V1" s="224" t="str">
+      <x:c r="V1" s="227" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="W1" s="224" t="str">
+      <x:c r="W1" s="227" t="str">
         <x:v>China_source_policy</x:v>
       </x:c>
-      <x:c r="X1" s="224" t="str">
+      <x:c r="X1" s="227" t="str">
         <x:v>Incoming_control</x:v>
       </x:c>
-      <x:c r="Y1" s="224" t="str">
+      <x:c r="Y1" s="227" t="str">
         <x:v>Program_scope</x:v>
       </x:c>
     </x:row>
@@ -55552,7 +55566,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b9bba641e74b92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re71fa95b132f43b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adopt PCB-MAIN 8-layer Rev.B EVT baseline
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1efdf6b8561447e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="Rd90521b2a91645ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Reea0dd1abd7540ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R3017a3b854c24ccd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R8340d9c1023249f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program 41" sheetId="6" r:id="R35d0b331236d436b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4e5fe1d010654038"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R8c56a37559b94ec4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rb48f76a9aafa4de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R4962d40fa7a24614"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R889b45f352b94ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program 41" sheetId="6" r:id="Rd3894cb7008548ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1986,10 +1986,10 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="G2" s="2" t="str">
-        <x:v>DIO-ASM-MAIN-REV-A</x:v>
+        <x:v>DIO-ASM-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="H2" s="2" t="str">
-        <x:v>6-layer PCBA build-to-print service scope</x:v>
+        <x:v>8-layer PCBA build-to-print service scope</x:v>
       </x:c>
       <x:c r="I2" s="2" t="str"/>
       <x:c r="J2" s="2" t="str">
@@ -2511,10 +2511,10 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="G9" s="2" t="str">
-        <x:v>DIO-PCB-MAIN-REV-A</x:v>
+        <x:v>DIO-PCB-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="H9" s="2" t="str">
-        <x:v>6-layer FR-4 110x75x1.6 mm build-to-print fabrication scope</x:v>
+        <x:v>8-layer FR-4 110x75x1.6 mm build-to-print fabrication scope</x:v>
       </x:c>
       <x:c r="I9" s="2" t="str"/>
       <x:c r="J9" s="2" t="str">
@@ -11414,7 +11414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcacf16b3d3744940"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd54d0811ca7e48bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11563,10 +11563,10 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="G2" s="2" t="str">
-        <x:v>DIO-ASM-MAIN-REV-A</x:v>
+        <x:v>DIO-ASM-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="H2" s="2" t="str">
-        <x:v>6-layer PCBA build-to-print service scope</x:v>
+        <x:v>8-layer PCBA build-to-print service scope</x:v>
       </x:c>
       <x:c r="I2" s="16" t="str">
         <x:v>1</x:v>
@@ -11650,10 +11650,10 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="G3" s="2" t="str">
-        <x:v>DIO-PCB-MAIN-REV-A</x:v>
+        <x:v>DIO-PCB-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="H3" s="2" t="str">
-        <x:v>6-layer FR-4 110x75x1.6 mm build-to-print fabrication scope</x:v>
+        <x:v>8-layer FR-4 110x75x1.6 mm build-to-print fabrication scope</x:v>
       </x:c>
       <x:c r="I3" s="16" t="str">
         <x:v>1</x:v>
@@ -37682,7 +37682,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f598f39f5a24813"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5bb1bce0c4a479f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38261,7 +38261,7 @@
         <x:v>Customer-selected standard PCBA service</x:v>
       </x:c>
       <x:c r="E12" s="81" t="str">
-        <x:v>DIO-PCBA-MAIN-EVT-A; JLC06161H-3313; SAC305 Type-4; 100 um stencil</x:v>
+        <x:v>DIO-PCBA-MAIN-EVT-B_JLC08161H-3313; SAC305 Type-4; 100 um stencil</x:v>
       </x:c>
       <x:c r="F12" s="82" t="str">
         <x:v>6</x:v>
@@ -38831,7 +38831,7 @@
         <x:v>JLCPCB or equivalent meeting EVT baseline</x:v>
       </x:c>
       <x:c r="E24" s="81" t="str">
-        <x:v>DIO-PCB-MAIN-EVT-A_JLC06161H-3313; 6-layer 1.6 mm order; ENIG; 1/0.5 oz; impedance +/-10 percent</x:v>
+        <x:v>DIO-PCB-MAIN-EVT-B_JLC08161H-3313; 8-layer 1.6 mm order; ENIG; 1/0.5 oz; impedance +/-10 percent</x:v>
       </x:c>
       <x:c r="F24" s="82" t="str">
         <x:v>6</x:v>
@@ -38861,7 +38861,7 @@
         <x:v>RFQ_REQUIRED</x:v>
       </x:c>
       <x:c r="S24" s="81" t="str">
-        <x:v>ALTERNATIVE QUOTATION TRACK ONLY; do not issue together with ASM-MAIN; upload only released Gerber drill IPC-356 and fabrication drawing after routing DRC CAM RF/SI and Review B; select JLC06161H-3313 controlled impedance and standard coupon/TDR when offered; stop on any checkout DFM or parser mismatch</x:v>
+        <x:v>ALTERNATIVE QUOTATION TRACK ONLY; do not issue together with ASM-MAIN; upload only released Gerber drill IPC-356 and fabrication drawing after routing DRC CAM RF/SI and Review B; select JLC08161H-3313 controlled impedance and standard coupon/TDR when offered; stop on any checkout DFM or parser mismatch</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="43.20000076293945" hidden="0" customHeight="1">
@@ -39062,7 +39062,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a15d8008f6c4ca8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2deef63792a1469c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39523,7 +39523,7 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="C13" s="134" t="str">
-        <x:v>DIO-ASM-MAIN-REV-A</x:v>
+        <x:v>DIO-ASM-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="D13" s="134" t="str">
         <x:v>PCBA</x:v>
@@ -39887,7 +39887,7 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="C20" s="134" t="str">
-        <x:v>DIO-PCB-MAIN-REV-A</x:v>
+        <x:v>DIO-PCB-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="D20" s="134" t="str">
         <x:v>Bare PCB</x:v>
@@ -46012,7 +46012,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8606e9aaabc346f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R864d6f1cab7d485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46145,10 +46145,10 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="G2" s="213" t="str">
-        <x:v>DIO-ASM-MAIN-REV-A</x:v>
+        <x:v>DIO-ASM-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="H2" s="213" t="str">
-        <x:v>6-layer PCBA build-to-print service scope</x:v>
+        <x:v>8-layer PCBA build-to-print service scope</x:v>
       </x:c>
       <x:c r="I2" s="213" t="str"/>
       <x:c r="J2" s="213" t="str">
@@ -46670,10 +46670,10 @@
         <x:v>Dioneya controlled design</x:v>
       </x:c>
       <x:c r="G9" s="213" t="str">
-        <x:v>DIO-PCB-MAIN-REV-A</x:v>
+        <x:v>DIO-PCB-MAIN-REV-B</x:v>
       </x:c>
       <x:c r="H9" s="213" t="str">
-        <x:v>6-layer FR-4 110x75x1.6 mm build-to-print fabrication scope</x:v>
+        <x:v>8-layer FR-4 110x75x1.6 mm build-to-print fabrication scope</x:v>
       </x:c>
       <x:c r="I9" s="213" t="str"/>
       <x:c r="J9" s="213" t="str">
@@ -55566,7 +55566,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re71fa95b132f43b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b106312a55b4581"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release EVT-PRE-20 manufacturing package
</commit_message>
<xml_diff>
--- a/hardware/EVT_PRE_20_BOM_REV_A.xlsx
+++ b/hardware/EVT_PRE_20_BOM_REV_A.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4e5fe1d010654038"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R8c56a37559b94ec4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rb48f76a9aafa4de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R4962d40fa7a24614"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R889b45f352b94ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program 41" sheetId="6" r:id="Rd3894cb7008548ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc09322392b45476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procurement" sheetId="2" r:id="R2a54f7476c474270"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering BOM" sheetId="3" r:id="Rf02bf8e9a3dc4dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ" sheetId="4" r:id="R27b0487bad10449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost estimate" sheetId="5" r:id="R54f421899fa940f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program 41" sheetId="6" r:id="R14ec984e756743d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3684,7 +3684,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W24" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X24" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -3836,7 +3836,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W26" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X26" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -3988,7 +3988,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W28" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X28" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -4142,7 +4142,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W30" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X30" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -4296,7 +4296,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W32" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X32" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -4677,7 +4677,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W37" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X37" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -4754,7 +4754,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W38" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X38" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -4831,7 +4831,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W39" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X39" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -4985,7 +4985,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W41" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X41" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -5293,7 +5293,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W45" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X45" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -5370,7 +5370,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W46" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X46" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -5447,7 +5447,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W47" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X47" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -5524,7 +5524,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W48" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X48" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -5832,7 +5832,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W52" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X52" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -5986,7 +5986,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W54" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X54" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6063,7 +6063,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W55" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X55" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6140,7 +6140,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W56" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X56" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6217,7 +6217,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W57" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X57" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6371,7 +6371,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W59" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X59" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6448,7 +6448,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W60" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X60" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6525,7 +6525,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W61" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X61" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6752,7 +6752,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W64" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X64" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6906,7 +6906,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W66" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X66" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -6983,7 +6983,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W67" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X67" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7060,7 +7060,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W68" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X68" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7214,7 +7214,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W70" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X70" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7291,7 +7291,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W71" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X71" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7368,7 +7368,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W72" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X72" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7445,7 +7445,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W73" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X73" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7522,7 +7522,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W74" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X74" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7599,7 +7599,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W75" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X75" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7753,7 +7753,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W77" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X77" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7830,7 +7830,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W78" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X78" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7907,7 +7907,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W79" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X79" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -7984,7 +7984,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W80" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X80" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -8061,7 +8061,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W81" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X81" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -8138,7 +8138,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W82" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X82" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -8515,7 +8515,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W87" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X87" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -8592,7 +8592,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W88" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X88" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -8669,7 +8669,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W89" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X89" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -9198,7 +9198,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W96" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X96" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -9275,7 +9275,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W97" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X97" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -9952,7 +9952,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W106" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X106" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10254,7 +10254,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W110" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X110" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10408,7 +10408,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W112" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X112" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10560,7 +10560,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W114" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X114" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10637,7 +10637,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W115" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X115" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10714,7 +10714,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W116" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X116" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -10791,7 +10791,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="W117" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="X117" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -11414,7 +11414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd54d0811ca7e48bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73f25dc0a80d4f63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16657,7 +16657,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U60" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V60" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -16746,7 +16746,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U61" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V61" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -16835,7 +16835,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U62" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V62" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -16924,7 +16924,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U63" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V63" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17013,7 +17013,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U64" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V64" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17102,7 +17102,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U65" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V65" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17191,7 +17191,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U66" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V66" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17280,7 +17280,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U67" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V67" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17369,7 +17369,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U68" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V68" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17458,7 +17458,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U69" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V69" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17547,7 +17547,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U70" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V70" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17636,7 +17636,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U71" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V71" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17725,7 +17725,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U72" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V72" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17814,7 +17814,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U73" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V73" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -17903,7 +17903,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U74" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V74" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18170,7 +18170,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U77" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V77" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18259,7 +18259,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U78" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V78" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18348,7 +18348,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U79" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V79" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18437,7 +18437,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U80" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V80" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18526,7 +18526,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U81" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V81" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18615,7 +18615,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U82" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V82" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18704,7 +18704,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U83" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V83" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18793,7 +18793,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U84" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V84" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18882,7 +18882,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U85" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V85" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -18971,7 +18971,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U86" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V86" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19060,7 +19060,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U87" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V87" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19149,7 +19149,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U88" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V88" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19238,7 +19238,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U89" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V89" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19327,7 +19327,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U90" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V90" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19416,7 +19416,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U91" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V91" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19505,7 +19505,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U92" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V92" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19594,7 +19594,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U93" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V93" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19683,7 +19683,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U94" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V94" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19772,7 +19772,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U95" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V95" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19861,7 +19861,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U96" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V96" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -19950,7 +19950,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U97" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V97" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20039,7 +20039,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U98" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V98" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20128,7 +20128,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U99" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V99" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20217,7 +20217,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U100" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V100" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20306,7 +20306,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U101" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V101" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20395,7 +20395,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U102" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V102" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20484,7 +20484,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U103" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V103" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20573,7 +20573,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U104" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V104" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20662,7 +20662,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U105" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V105" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20751,7 +20751,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U106" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V106" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20840,7 +20840,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U107" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V107" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -20929,7 +20929,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U108" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V108" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -21018,7 +21018,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U109" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V109" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -21107,7 +21107,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U110" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V110" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -21196,7 +21196,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U111" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V111" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -21285,7 +21285,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U112" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V112" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -21908,7 +21908,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U119" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V119" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -21997,7 +21997,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U120" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V120" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22086,7 +22086,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U121" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V121" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22175,7 +22175,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U122" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V122" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22264,7 +22264,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U123" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V123" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22353,7 +22353,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U124" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V124" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22442,7 +22442,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U125" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V125" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22531,7 +22531,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U126" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V126" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22620,7 +22620,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U127" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V127" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22887,7 +22887,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U130" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V130" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -22976,7 +22976,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U131" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V131" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23065,7 +23065,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U132" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V132" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23154,7 +23154,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U133" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V133" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23243,7 +23243,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U134" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V134" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23332,7 +23332,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U135" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V135" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23421,7 +23421,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U136" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V136" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23510,7 +23510,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U137" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V137" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23777,7 +23777,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U140" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V140" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23866,7 +23866,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U141" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V141" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -23955,7 +23955,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U142" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V142" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24133,7 +24133,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U144" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V144" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24311,7 +24311,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U146" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V146" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24400,7 +24400,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U147" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V147" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24489,7 +24489,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U148" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V148" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24578,7 +24578,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U149" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V149" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24667,7 +24667,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U150" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V150" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24756,7 +24756,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U151" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V151" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24845,7 +24845,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U152" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V152" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -24934,7 +24934,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U153" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V153" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25023,7 +25023,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U154" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V154" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25112,7 +25112,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U155" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V155" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25201,7 +25201,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U156" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V156" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25290,7 +25290,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U157" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V157" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25379,7 +25379,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U158" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V158" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25468,7 +25468,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U159" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V159" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25557,7 +25557,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U160" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V160" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25646,7 +25646,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U161" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V161" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25735,7 +25735,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U162" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V162" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25824,7 +25824,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U163" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V163" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -25913,7 +25913,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U164" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V164" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26002,7 +26002,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U165" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V165" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26091,7 +26091,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U166" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V166" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26180,7 +26180,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U167" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V167" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26269,7 +26269,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U168" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V168" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26358,7 +26358,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U169" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V169" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26447,7 +26447,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U170" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V170" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26536,7 +26536,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U171" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V171" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26625,7 +26625,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U172" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V172" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26714,7 +26714,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U173" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V173" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26803,7 +26803,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U174" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V174" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26892,7 +26892,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U175" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V175" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -26981,7 +26981,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U176" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V176" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27070,7 +27070,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U177" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V177" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27159,7 +27159,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U178" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V178" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27248,7 +27248,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U179" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V179" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27337,7 +27337,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U180" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V180" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27426,7 +27426,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U181" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V181" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27515,7 +27515,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U182" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V182" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27604,7 +27604,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U183" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V183" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27693,7 +27693,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U184" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V184" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27782,7 +27782,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U185" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V185" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27871,7 +27871,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U186" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V186" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -27960,7 +27960,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U187" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V187" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28049,7 +28049,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U188" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V188" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28138,7 +28138,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U189" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V189" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28227,7 +28227,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U190" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V190" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28316,7 +28316,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U191" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V191" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28405,7 +28405,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U192" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V192" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28494,7 +28494,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U193" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V193" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28583,7 +28583,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U194" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V194" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28672,7 +28672,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U195" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V195" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28761,7 +28761,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U196" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V196" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28850,7 +28850,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U197" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V197" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -28939,7 +28939,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U198" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V198" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29028,7 +29028,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U199" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V199" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29117,7 +29117,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U200" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V200" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29206,7 +29206,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U201" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V201" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29295,7 +29295,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U202" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V202" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29384,7 +29384,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U203" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V203" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29473,7 +29473,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U204" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V204" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29562,7 +29562,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U205" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V205" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29651,7 +29651,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U206" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V206" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29740,7 +29740,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U207" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V207" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29829,7 +29829,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U208" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V208" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -29918,7 +29918,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U209" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V209" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30007,7 +30007,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U210" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V210" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30096,7 +30096,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U211" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V211" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30185,7 +30185,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U212" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V212" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30274,7 +30274,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U213" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V213" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30363,7 +30363,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U214" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V214" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30452,7 +30452,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U215" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V215" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30541,7 +30541,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U216" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V216" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30630,7 +30630,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U217" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V217" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30719,7 +30719,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U218" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V218" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30808,7 +30808,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U219" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V219" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30897,7 +30897,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U220" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V220" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -30986,7 +30986,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U221" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V221" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31075,7 +31075,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U222" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V222" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31164,7 +31164,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U223" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V223" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31253,7 +31253,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U224" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V224" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31342,7 +31342,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U225" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V225" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31431,7 +31431,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U226" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V226" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31520,7 +31520,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U227" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V227" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31609,7 +31609,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U228" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V228" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31698,7 +31698,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U229" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V229" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31787,7 +31787,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U230" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V230" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31876,7 +31876,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U231" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V231" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -31965,7 +31965,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U232" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V232" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32054,7 +32054,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U233" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V233" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32143,7 +32143,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U234" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V234" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32232,7 +32232,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U235" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V235" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32321,7 +32321,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U236" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V236" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32499,7 +32499,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U238" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V238" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32588,7 +32588,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U239" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V239" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32677,7 +32677,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U240" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V240" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32766,7 +32766,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U241" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V241" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32855,7 +32855,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U242" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V242" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -32944,7 +32944,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U243" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V243" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33033,7 +33033,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U244" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V244" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33122,7 +33122,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U245" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V245" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33211,7 +33211,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U246" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V246" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33300,7 +33300,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U247" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V247" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33389,7 +33389,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U248" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V248" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33478,7 +33478,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U249" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V249" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33567,7 +33567,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U250" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V250" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33656,7 +33656,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U251" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V251" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33745,7 +33745,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U252" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V252" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33834,7 +33834,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U253" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V253" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -33923,7 +33923,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U254" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V254" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34012,7 +34012,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U255" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V255" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34101,7 +34101,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U256" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V256" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34190,7 +34190,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U257" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V257" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34279,7 +34279,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U258" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V258" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34368,7 +34368,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U259" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V259" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34457,7 +34457,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U260" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V260" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34546,7 +34546,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U261" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V261" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34635,7 +34635,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U262" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V262" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34724,7 +34724,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U263" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V263" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34813,7 +34813,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U264" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V264" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34902,7 +34902,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U265" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V265" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -34991,7 +34991,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U266" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V266" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -35080,7 +35080,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U267" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V267" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -35169,7 +35169,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U268" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V268" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -35258,7 +35258,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U269" s="14" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V269" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36132,7 +36132,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U279" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V279" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36221,7 +36221,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U280" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V280" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36577,7 +36577,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U284" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V284" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36666,7 +36666,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U285" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V285" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36755,7 +36755,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U286" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V286" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36844,7 +36844,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U287" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V287" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -36933,7 +36933,7 @@
         <x:v>COMMON</x:v>
       </x:c>
       <x:c r="U288" s="14" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="V288" s="17" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -37682,7 +37682,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5bb1bce0c4a479f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R471e5759718645dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39062,7 +39062,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2deef63792a1469c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04432e0152c54b36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46012,7 +46012,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R864d6f1cab7d485f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4230bae48f064b6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47840,7 +47840,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V24" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W24" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -47992,7 +47992,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V26" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W26" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -48144,7 +48144,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V28" s="213" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W28" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -48298,7 +48298,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V30" s="213" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W30" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -48452,7 +48452,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V32" s="213" t="str">
-        <x:v>LOCKED_CANDIDATE_PENDING_DERATING</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W32" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -48833,7 +48833,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V37" s="213" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W37" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -48910,7 +48910,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V38" s="213" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W38" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -48987,7 +48987,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V39" s="213" t="str">
-        <x:v>LOCKED_CANDIDATE</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W39" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -49141,7 +49141,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V41" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W41" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -49449,7 +49449,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V45" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W45" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -49526,7 +49526,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V46" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W46" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -49603,7 +49603,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V47" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W47" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -49680,7 +49680,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V48" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W48" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -49988,7 +49988,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V52" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W52" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50142,7 +50142,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V54" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W54" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50219,7 +50219,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V55" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W55" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50296,7 +50296,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V56" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W56" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50373,7 +50373,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V57" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W57" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50527,7 +50527,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V59" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W59" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50604,7 +50604,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V60" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W60" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50681,7 +50681,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V61" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W61" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -50908,7 +50908,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V64" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W64" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51062,7 +51062,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V66" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W66" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51139,7 +51139,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V67" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W67" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51216,7 +51216,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V68" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W68" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51370,7 +51370,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V70" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W70" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51447,7 +51447,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V71" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W71" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51524,7 +51524,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V72" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W72" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51601,7 +51601,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V73" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W73" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51678,7 +51678,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V74" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W74" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51755,7 +51755,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V75" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W75" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51909,7 +51909,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V77" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W77" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -51986,7 +51986,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V78" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W78" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52063,7 +52063,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V79" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W79" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52140,7 +52140,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V80" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W80" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52217,7 +52217,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V81" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W81" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52294,7 +52294,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V82" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W82" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52671,7 +52671,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V87" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W87" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52748,7 +52748,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V88" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W88" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -52825,7 +52825,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V89" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W89" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -53354,7 +53354,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V96" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W96" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -53431,7 +53431,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V97" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W97" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54108,7 +54108,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V106" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W106" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54410,7 +54410,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V110" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W110" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54564,7 +54564,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V112" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W112" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54716,7 +54716,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V114" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W114" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54793,7 +54793,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V115" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W115" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54870,7 +54870,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V116" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W116" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -54947,7 +54947,7 @@
         <x:v>CONTROLLED_PENDING_VERIFICATION</x:v>
       </x:c>
       <x:c r="V117" s="213" t="str">
-        <x:v>SELECTED_PENDING_REVIEW_A</x:v>
+        <x:v>CONTROLLED_EVT_ENGINEERING_ACCEPTED_PHYSICAL_VALIDATION_AT_EVT</x:v>
       </x:c>
       <x:c r="W117" s="213" t="str">
         <x:v>Authorized or traceable tier-1 channel</x:v>
@@ -55566,7 +55566,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b106312a55b4581"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0359fa3d458428e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>